<commit_message>
update C.13 + Giao thuc
</commit_message>
<xml_diff>
--- a/Kỹ Thuật lập trình/C/13. EMBEDDED SYSTEMS PROGRAMMING.xlsx
+++ b/Kỹ Thuật lập trình/C/13. EMBEDDED SYSTEMS PROGRAMMING.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="3"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Mục lục" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5759" uniqueCount="4111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5775" uniqueCount="4126">
   <si>
     <t>🎯 EMBEDDED SYSTEMS PROGRAMMING</t>
   </si>
@@ -12122,9 +12122,6 @@
     <t>6. Communication Protocols</t>
   </si>
   <si>
-    <t>6.1 UART Programming</t>
-  </si>
-  <si>
     <t>6.1.1 UART Initialization</t>
   </si>
   <si>
@@ -12326,9 +12323,6 @@
     <t xml:space="preserve">    UART_TransmitString((char*)&amp;packet);</t>
   </si>
   <si>
-    <t>6.2 SPI Communication</t>
-  </si>
-  <si>
     <t>6.2.1 SPI Master Configuration</t>
   </si>
   <si>
@@ -12516,9 +12510,6 @@
   </si>
   <si>
     <t xml:space="preserve">    while (SPI1-&gt;SR &amp; SPI_SR_BSY);</t>
-  </si>
-  <si>
-    <t>6.3 I2C Communication</t>
   </si>
   <si>
     <t>6.3.1 I2C Master Implementation</t>
@@ -12855,12 +12846,66 @@
   <si>
     <t xml:space="preserve">    uint8_t end;       // 0x55</t>
   </si>
+  <si>
+    <t>=&gt; UART Hardware thực hiện đúng nhiệm vụ của tầng vật lý</t>
+  </si>
+  <si>
+    <t>sau khi gom được các bit Data từ tầng vật lý, nhiệm vụ tiếp theo đọc như nào sẽ nhờ software.</t>
+  </si>
+  <si>
+    <t>=&gt; UART Software thực hiện phân tích Data theo cách lập trình viên định nghĩa.</t>
+  </si>
+  <si>
+    <t>6.2 SPI Communication (Serial Peripheral Interface)</t>
+  </si>
+  <si>
+    <t>serial : truyền dữ liệu từng bit nối tiếp ( không phải song song )</t>
+  </si>
+  <si>
+    <t>6.1 UART Programming (Universal Asynchronous Receiver – Transmitter)</t>
+  </si>
+  <si>
+    <t>MOSI :  Data: Master Out, Slave in</t>
+  </si>
+  <si>
+    <t>MISO : Data: Master in, Slave out</t>
+  </si>
+  <si>
+    <t>SCK : Serial Clock (do Master tạo xung)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cách thức hoạt động : Master gửi Data (có thể có chủ đích hoặc bất kỳ)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">xuống Slave được chọn để đồng bộ tín hiệu và nhận data về </t>
+  </si>
+  <si>
+    <t>=&gt; số thiết bị kết nối bị giới hạn</t>
+  </si>
+  <si>
+    <t>Đường SS (Slave Select): chọn Slave (mỗi Slave lại cần 1 dây SS nối với chân cs của Slave )</t>
+  </si>
+  <si>
+    <t>Giao tiếp bất đồng bộ</t>
+  </si>
+  <si>
+    <t>Giao tiếp đồng bộ</t>
+  </si>
+  <si>
+    <t>6.3 I2C Communication (Inter-Integrated Circuit)</t>
+  </si>
+  <si>
+    <t>Inter-Integrated Circuit nghĩa là: chuẩn giao tiếp nối tiếp để các IC nói chuyện trực tiếp với nhau trên cùng một bo mạch (PCB).</t>
+  </si>
+  <si>
+    <t>Full-duplex (gửi và nhận cùng lúc).</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -12960,13 +13005,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
       <color theme="1"/>
@@ -12985,8 +13023,27 @@
       <name val="Arial Unicode MS"/>
       <charset val="163"/>
     </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="163"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="163"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -13047,8 +13104,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="14">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -13193,11 +13256,48 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -13283,17 +13383,17 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -13324,6 +13424,25 @@
     <xf numFmtId="0" fontId="6" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -13980,6 +14099,542 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>45</xdr:col>
+      <xdr:colOff>66675</xdr:colOff>
+      <xdr:row>167</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>66</xdr:col>
+      <xdr:colOff>127000</xdr:colOff>
+      <xdr:row>182</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Picture 6" descr="A diagram of a computer&#10;&#10;Description automatically generated with medium confidence"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10782300" y="30594300"/>
+          <a:ext cx="5060950" cy="2781300"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>45</xdr:col>
+      <xdr:colOff>66675</xdr:colOff>
+      <xdr:row>182</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>66</xdr:col>
+      <xdr:colOff>133350</xdr:colOff>
+      <xdr:row>198</xdr:row>
+      <xdr:rowOff>104775</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Picture 7" descr="A white paper with black text and numbers&#10;&#10;Description automatically generated"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10782300" y="33385125"/>
+          <a:ext cx="5067300" cy="2876550"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>45</xdr:col>
+      <xdr:colOff>85724</xdr:colOff>
+      <xdr:row>198</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>66</xdr:col>
+      <xdr:colOff>104774</xdr:colOff>
+      <xdr:row>208</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11" name="Picture 10" descr="A screenshot of a computer&#10;&#10;Description automatically generated"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10801349" y="36280725"/>
+          <a:ext cx="5019675" cy="1819275"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>33</xdr:col>
+      <xdr:colOff>200025</xdr:colOff>
+      <xdr:row>203</xdr:row>
+      <xdr:rowOff>128588</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>45</xdr:col>
+      <xdr:colOff>85724</xdr:colOff>
+      <xdr:row>210</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="6" name="Straight Arrow Connector 5"/>
+        <xdr:cNvCxnSpPr>
+          <a:endCxn id="11" idx="1"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="8058150" y="37190363"/>
+          <a:ext cx="2743199" cy="1309687"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>66675</xdr:colOff>
+      <xdr:row>177</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>49532</xdr:colOff>
+      <xdr:row>214</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="14" name="Straight Arrow Connector 13"/>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6019800" y="32499300"/>
+          <a:ext cx="1411607" cy="6659880"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>240</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>180975</xdr:colOff>
+      <xdr:row>243</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="19" name="Straight Arrow Connector 18"/>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="1914525" y="44081700"/>
+          <a:ext cx="2076450" cy="476250"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>45</xdr:col>
+      <xdr:colOff>180975</xdr:colOff>
+      <xdr:row>264</xdr:row>
+      <xdr:rowOff>104775</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>69</xdr:col>
+      <xdr:colOff>93345</xdr:colOff>
+      <xdr:row>276</xdr:row>
+      <xdr:rowOff>66040</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="21" name="Picture 20"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="10896600" y="48491775"/>
+          <a:ext cx="5627370" cy="2132965"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>53</xdr:col>
+      <xdr:colOff>114300</xdr:colOff>
+      <xdr:row>203</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>61</xdr:col>
+      <xdr:colOff>66675</xdr:colOff>
+      <xdr:row>211</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="23" name="Straight Arrow Connector 22"/>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="12734925" y="37109400"/>
+          <a:ext cx="1857375" cy="1466850"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>43</xdr:col>
+      <xdr:colOff>200025</xdr:colOff>
+      <xdr:row>268</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>50</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>276</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="25" name="Straight Arrow Connector 24"/>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1">
+          <a:off x="10439400" y="49253775"/>
+          <a:ext cx="1543050" cy="1457325"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>104775</xdr:colOff>
+      <xdr:row>305</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>306</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="27" name="Straight Arrow Connector 26"/>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="2486025" y="55987950"/>
+          <a:ext cx="609600" cy="180975"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>54</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>182</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>61</xdr:col>
+      <xdr:colOff>28575</xdr:colOff>
+      <xdr:row>213</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="29" name="Straight Arrow Connector 28"/>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="12877800" y="33251775"/>
+          <a:ext cx="1676400" cy="5715000"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>46</xdr:col>
+      <xdr:colOff>66675</xdr:colOff>
+      <xdr:row>269</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>57</xdr:col>
+      <xdr:colOff>190500</xdr:colOff>
+      <xdr:row>279</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="31" name="Straight Arrow Connector 30"/>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1">
+          <a:off x="11020425" y="49444275"/>
+          <a:ext cx="2743200" cy="1704975"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -14247,10 +14902,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B1:AC14"/>
-  <sheetFormatPr defaultColWidth="3.09765625" defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultColWidth="3.125" defaultRowHeight="14.25"/>
   <sheetData>
-    <row r="1" spans="2:29" ht="14.4" thickBot="1"/>
-    <row r="2" spans="2:29" ht="23.4" thickBot="1">
+    <row r="1" spans="2:29" ht="15" thickBot="1"/>
+    <row r="2" spans="2:29" ht="24" thickBot="1">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -14275,7 +14930,7 @@
       <c r="U2" s="2"/>
       <c r="V2" s="3"/>
     </row>
-    <row r="3" spans="2:29" ht="17.399999999999999">
+    <row r="3" spans="2:29" ht="17.25">
       <c r="B3" s="4" t="s">
         <v>1</v>
       </c>
@@ -14286,7 +14941,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="2:29">
+    <row r="4" spans="2:29" ht="15">
       <c r="B4" s="5" t="s">
         <v>4</v>
       </c>
@@ -14346,7 +15001,7 @@
       <c r="P9" s="5"/>
       <c r="AC9" s="5"/>
     </row>
-    <row r="10" spans="2:29">
+    <row r="10" spans="2:29" ht="15">
       <c r="B10" s="5" t="s">
         <v>19</v>
       </c>
@@ -14409,17 +15064,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:CM968"/>
-  <sheetFormatPr defaultColWidth="3.09765625" defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultColWidth="3.125" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="16384" width="3.09765625" style="9"/>
+    <col min="1" max="16384" width="3.125" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:65" s="14" customFormat="1" ht="14.4" thickBot="1">
+    <row r="1" spans="1:65" s="14" customFormat="1" ht="15.75" thickBot="1">
       <c r="A1" s="13" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:65">
+    <row r="2" spans="1:65" ht="15">
       <c r="A2" s="16" t="s">
         <v>35</v>
       </c>
@@ -14450,7 +15105,7 @@
       <c r="BL2" s="17"/>
       <c r="BM2" s="17"/>
     </row>
-    <row r="3" spans="1:65">
+    <row r="3" spans="1:65" ht="15">
       <c r="A3" s="8" t="s">
         <v>36</v>
       </c>
@@ -14497,7 +15152,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="5" spans="1:65">
+    <row r="5" spans="1:65" ht="15">
       <c r="A5" s="11" t="s">
         <v>1404</v>
       </c>
@@ -14581,7 +15236,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="8" spans="1:65">
+    <row r="8" spans="1:65" ht="15">
       <c r="A8" s="10" t="s">
         <v>38</v>
       </c>
@@ -14683,7 +15338,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="11" spans="1:65">
+    <row r="11" spans="1:65" ht="15">
       <c r="A11" s="10" t="s">
         <v>41</v>
       </c>
@@ -14760,7 +15415,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="14" spans="1:65">
+    <row r="14" spans="1:65" ht="15">
       <c r="A14" s="10" t="s">
         <v>43</v>
       </c>
@@ -14877,7 +15532,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="17" spans="1:64">
+    <row r="17" spans="1:64" ht="15">
       <c r="A17" s="10" t="s">
         <v>46</v>
       </c>
@@ -14984,7 +15639,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="20" spans="1:64">
+    <row r="20" spans="1:64" ht="15">
       <c r="A20" s="10" t="s">
         <v>48</v>
       </c>
@@ -15121,13 +15776,13 @@
         <v>135</v>
       </c>
     </row>
-    <row r="26" spans="1:64">
+    <row r="26" spans="1:64" ht="15">
       <c r="AC26" s="8" t="s">
         <v>96</v>
       </c>
       <c r="BG26" s="11"/>
     </row>
-    <row r="27" spans="1:64">
+    <row r="27" spans="1:64" ht="15">
       <c r="A27" s="8" t="s">
         <v>51</v>
       </c>
@@ -15157,7 +15812,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="30" spans="1:64">
+    <row r="30" spans="1:64" ht="15">
       <c r="A30" s="10" t="s">
         <v>54</v>
       </c>
@@ -15426,7 +16081,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="62" spans="1:55">
+    <row r="62" spans="1:55" ht="15">
       <c r="A62" s="16" t="s">
         <v>152</v>
       </c>
@@ -15448,7 +16103,7 @@
       <c r="AF62" s="17"/>
       <c r="AG62" s="17"/>
     </row>
-    <row r="63" spans="1:55">
+    <row r="63" spans="1:55" ht="15">
       <c r="A63" s="44" t="s">
         <v>153</v>
       </c>
@@ -15716,7 +16371,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="74" spans="1:49">
+    <row r="74" spans="1:49" ht="15">
       <c r="A74" s="8" t="s">
         <v>161</v>
       </c>
@@ -15960,7 +16615,7 @@
       </c>
       <c r="AW98" s="11"/>
     </row>
-    <row r="99" spans="1:49">
+    <row r="99" spans="1:49" ht="15">
       <c r="A99" s="8" t="s">
         <v>177</v>
       </c>
@@ -16134,13 +16789,13 @@
         <v>265</v>
       </c>
     </row>
-    <row r="118" spans="1:73" ht="14.4" thickBot="1"/>
-    <row r="119" spans="1:73" s="14" customFormat="1" ht="14.4" thickBot="1">
+    <row r="118" spans="1:73" ht="15" thickBot="1"/>
+    <row r="119" spans="1:73" s="14" customFormat="1" ht="15.75" thickBot="1">
       <c r="A119" s="13" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="120" spans="1:73">
+    <row r="120" spans="1:73" ht="15">
       <c r="A120" s="16" t="s">
         <v>267</v>
       </c>
@@ -16175,7 +16830,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="121" spans="1:73">
+    <row r="121" spans="1:73" ht="15">
       <c r="A121" s="43" t="s">
         <v>268</v>
       </c>
@@ -16195,7 +16850,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="122" spans="1:73">
+    <row r="122" spans="1:73" ht="15">
       <c r="A122" s="42" t="s">
         <v>269</v>
       </c>
@@ -16235,7 +16890,7 @@
         <v>426</v>
       </c>
     </row>
-    <row r="125" spans="1:73">
+    <row r="125" spans="1:73" ht="15">
       <c r="A125" s="42" t="s">
         <v>271</v>
       </c>
@@ -16261,7 +16916,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="127" spans="1:73">
+    <row r="127" spans="1:73" ht="15">
       <c r="A127" s="42" t="s">
         <v>273</v>
       </c>
@@ -16303,7 +16958,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="130" spans="1:73">
+    <row r="130" spans="1:73" ht="15">
       <c r="A130" s="42" t="s">
         <v>275</v>
       </c>
@@ -16343,7 +16998,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="133" spans="1:73">
+    <row r="133" spans="1:73" ht="15">
       <c r="A133" s="42" t="s">
         <v>277</v>
       </c>
@@ -16636,7 +17291,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="155" spans="1:73">
+    <row r="155" spans="1:73" ht="15">
       <c r="A155" s="10" t="s">
         <v>292</v>
       </c>
@@ -16743,7 +17398,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="163" spans="1:73">
+    <row r="163" spans="1:73" ht="15">
       <c r="A163" s="10" t="s">
         <v>298</v>
       </c>
@@ -16839,7 +17494,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="170" spans="1:73">
+    <row r="170" spans="1:73" ht="15">
       <c r="A170" s="10" t="s">
         <v>46</v>
       </c>
@@ -16864,7 +17519,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="172" spans="1:73">
+    <row r="172" spans="1:73" ht="15">
       <c r="A172" s="44" t="s">
         <v>303</v>
       </c>
@@ -17151,7 +17806,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="189" spans="1:73">
+    <row r="189" spans="1:73" ht="15">
       <c r="A189" s="42" t="s">
         <v>316</v>
       </c>
@@ -17352,17 +18007,17 @@
         <v>490</v>
       </c>
     </row>
-    <row r="218" spans="1:76" ht="14.4" thickBot="1">
+    <row r="218" spans="1:76" ht="15" thickBot="1">
       <c r="BU218" s="10" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="219" spans="1:76" s="14" customFormat="1" ht="14.4" thickBot="1">
+    <row r="219" spans="1:76" s="14" customFormat="1" ht="15.75" thickBot="1">
       <c r="A219" s="13" t="s">
         <v>491</v>
       </c>
     </row>
-    <row r="220" spans="1:76">
+    <row r="220" spans="1:76" ht="15">
       <c r="A220" s="16" t="s">
         <v>492</v>
       </c>
@@ -17493,7 +18148,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="226" spans="1:91">
+    <row r="226" spans="1:91" ht="15">
       <c r="A226" s="11"/>
       <c r="Y226" s="10" t="s">
         <v>520</v>
@@ -17663,7 +18318,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="236" spans="1:91">
+    <row r="236" spans="1:91" ht="15">
       <c r="A236" s="11"/>
       <c r="Y236" s="10" t="s">
         <v>46</v>
@@ -17809,7 +18464,7 @@
       </c>
       <c r="BN245" s="11"/>
     </row>
-    <row r="246" spans="1:76">
+    <row r="246" spans="1:76" ht="15">
       <c r="A246" s="10" t="s">
         <v>509</v>
       </c>
@@ -17884,7 +18539,7 @@
       <c r="BW250" s="18"/>
       <c r="BX250" s="18"/>
     </row>
-    <row r="251" spans="1:76">
+    <row r="251" spans="1:76" ht="15">
       <c r="A251" s="10" t="s">
         <v>514</v>
       </c>
@@ -18326,7 +18981,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="272" spans="24:76">
+    <row r="272" spans="24:76" ht="15">
       <c r="Y272" s="10" t="s">
         <v>542</v>
       </c>
@@ -18348,7 +19003,7 @@
         <v>642</v>
       </c>
     </row>
-    <row r="273" spans="25:66">
+    <row r="273" spans="25:66" ht="15">
       <c r="Y273" s="10" t="s">
         <v>543</v>
       </c>
@@ -18370,7 +19025,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="274" spans="25:66">
+    <row r="274" spans="25:66" ht="15">
       <c r="Y274" s="11"/>
       <c r="AS274" s="10" t="s">
         <v>605</v>
@@ -18886,17 +19541,17 @@
         <v>570</v>
       </c>
     </row>
-    <row r="320" spans="25:25" ht="14.4" thickBot="1">
+    <row r="320" spans="25:25" ht="15" thickBot="1">
       <c r="Y320" s="10" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="321" spans="1:59" s="14" customFormat="1" ht="14.4" thickBot="1">
+    <row r="321" spans="1:59" s="14" customFormat="1" ht="15.75" thickBot="1">
       <c r="A321" s="13" t="s">
         <v>662</v>
       </c>
     </row>
-    <row r="322" spans="1:59">
+    <row r="322" spans="1:59" ht="15">
       <c r="A322" s="8" t="s">
         <v>663</v>
       </c>
@@ -20209,7 +20864,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="462" spans="1:61">
+    <row r="462" spans="1:61" ht="15">
       <c r="A462" s="8" t="s">
         <v>904</v>
       </c>
@@ -22244,17 +22899,17 @@
         <v>1170</v>
       </c>
     </row>
-    <row r="700" spans="1:51" ht="14.4" thickBot="1">
+    <row r="700" spans="1:51" ht="15" thickBot="1">
       <c r="AF700" s="10" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="701" spans="1:51" s="14" customFormat="1" ht="14.4" thickBot="1">
+    <row r="701" spans="1:51" s="14" customFormat="1" ht="15.75" thickBot="1">
       <c r="A701" s="13" t="s">
         <v>1246</v>
       </c>
     </row>
-    <row r="702" spans="1:51">
+    <row r="702" spans="1:51" ht="15">
       <c r="A702" s="8" t="s">
         <v>1247</v>
       </c>
@@ -23162,58 +23817,58 @@
         <v>46</v>
       </c>
     </row>
-    <row r="949" spans="1:1">
+    <row r="949" spans="1:1" ht="15">
       <c r="A949" s="8"/>
     </row>
-    <row r="951" spans="1:1">
+    <row r="951" spans="1:1" ht="15">
       <c r="A951" s="8"/>
     </row>
     <row r="952" spans="1:1">
       <c r="A952" s="12"/>
     </row>
-    <row r="953" spans="1:1">
+    <row r="953" spans="1:1" ht="15">
       <c r="A953" s="7"/>
     </row>
     <row r="954" spans="1:1">
       <c r="A954" s="12"/>
     </row>
-    <row r="955" spans="1:1">
+    <row r="955" spans="1:1" ht="15">
       <c r="A955" s="7"/>
     </row>
     <row r="956" spans="1:1">
       <c r="A956" s="12"/>
     </row>
-    <row r="957" spans="1:1">
+    <row r="957" spans="1:1" ht="15">
       <c r="A957" s="7"/>
     </row>
     <row r="958" spans="1:1">
       <c r="A958" s="12"/>
     </row>
-    <row r="959" spans="1:1">
+    <row r="959" spans="1:1" ht="15">
       <c r="A959" s="7"/>
     </row>
     <row r="960" spans="1:1">
       <c r="A960" s="12"/>
     </row>
-    <row r="961" spans="1:1">
+    <row r="961" spans="1:1" ht="15">
       <c r="A961" s="7"/>
     </row>
-    <row r="963" spans="1:1">
+    <row r="963" spans="1:1" ht="15">
       <c r="A963" s="8"/>
     </row>
     <row r="964" spans="1:1">
       <c r="A964" s="12"/>
     </row>
-    <row r="965" spans="1:1">
+    <row r="965" spans="1:1" ht="15">
       <c r="A965" s="7"/>
     </row>
-    <row r="966" spans="1:1">
+    <row r="966" spans="1:1" ht="15">
       <c r="A966" s="7"/>
     </row>
-    <row r="967" spans="1:1">
+    <row r="967" spans="1:1" ht="15">
       <c r="A967" s="7"/>
     </row>
-    <row r="968" spans="1:1">
+    <row r="968" spans="1:1" ht="15">
       <c r="A968" s="7"/>
     </row>
   </sheetData>
@@ -23226,17 +23881,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:CG1090"/>
-  <sheetFormatPr defaultColWidth="3.09765625" defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultColWidth="3.125" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="16384" width="3.09765625" style="9"/>
+    <col min="1" max="16384" width="3.125" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:71" s="14" customFormat="1" ht="14.4" thickBot="1">
+    <row r="1" spans="1:71" s="14" customFormat="1" ht="15.75" thickBot="1">
       <c r="A1" s="13" t="s">
         <v>2791</v>
       </c>
     </row>
-    <row r="2" spans="1:71">
+    <row r="2" spans="1:71" ht="15">
       <c r="A2" s="16" t="s">
         <v>2792</v>
       </c>
@@ -23292,7 +23947,7 @@
       <c r="BR2" s="17"/>
       <c r="BS2" s="17"/>
     </row>
-    <row r="3" spans="1:71">
+    <row r="3" spans="1:71" ht="15">
       <c r="A3" s="49" t="s">
         <v>3274</v>
       </c>
@@ -23320,7 +23975,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="5" spans="1:71">
+    <row r="5" spans="1:71" ht="15">
       <c r="A5" s="7" t="s">
         <v>3254</v>
       </c>
@@ -23332,7 +23987,7 @@
         <v>2391</v>
       </c>
     </row>
-    <row r="6" spans="1:71">
+    <row r="6" spans="1:71" ht="15">
       <c r="A6" s="7" t="s">
         <v>3255</v>
       </c>
@@ -23346,7 +24001,7 @@
         <v>2392</v>
       </c>
     </row>
-    <row r="7" spans="1:71">
+    <row r="7" spans="1:71" ht="15">
       <c r="A7" s="7" t="s">
         <v>3256</v>
       </c>
@@ -23358,7 +24013,7 @@
         <v>2393</v>
       </c>
     </row>
-    <row r="8" spans="1:71">
+    <row r="8" spans="1:71" ht="15">
       <c r="A8" s="7" t="s">
         <v>3257</v>
       </c>
@@ -23372,7 +24027,7 @@
         <v>2394</v>
       </c>
     </row>
-    <row r="9" spans="1:71">
+    <row r="9" spans="1:71" ht="15">
       <c r="A9" s="7" t="s">
         <v>3258</v>
       </c>
@@ -23397,7 +24052,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="11" spans="1:71">
+    <row r="11" spans="1:71" ht="15">
       <c r="A11" s="16" t="s">
         <v>2793</v>
       </c>
@@ -23753,17 +24408,17 @@
         <v>2417</v>
       </c>
     </row>
-    <row r="44" spans="1:62" ht="14.4" thickBot="1">
+    <row r="44" spans="1:62" ht="15" thickBot="1">
       <c r="BJ44" s="10" t="s">
         <v>2418</v>
       </c>
     </row>
-    <row r="45" spans="1:62" s="14" customFormat="1" ht="14.4" thickBot="1">
+    <row r="45" spans="1:62" s="14" customFormat="1" ht="15.75" thickBot="1">
       <c r="A45" s="13" t="s">
         <v>2419</v>
       </c>
     </row>
-    <row r="46" spans="1:62">
+    <row r="46" spans="1:62" ht="15">
       <c r="A46" s="16" t="s">
         <v>2420</v>
       </c>
@@ -23792,7 +24447,7 @@
       <c r="AD46" s="17"/>
       <c r="AE46" s="17"/>
     </row>
-    <row r="47" spans="1:62">
+    <row r="47" spans="1:62" ht="15">
       <c r="A47" s="52" t="s">
         <v>3282</v>
       </c>
@@ -23822,7 +24477,7 @@
       </c>
       <c r="AR47" s="18"/>
     </row>
-    <row r="48" spans="1:62">
+    <row r="48" spans="1:62" ht="15">
       <c r="A48" s="18" t="s">
         <v>3276</v>
       </c>
@@ -23852,7 +24507,7 @@
       </c>
       <c r="AR48" s="18"/>
     </row>
-    <row r="49" spans="1:43">
+    <row r="49" spans="1:43" ht="15">
       <c r="A49" s="8" t="s">
         <v>2421</v>
       </c>
@@ -23863,7 +24518,7 @@
         <v>2471</v>
       </c>
     </row>
-    <row r="50" spans="1:43">
+    <row r="50" spans="1:43" ht="15">
       <c r="A50" s="7" t="s">
         <v>3259</v>
       </c>
@@ -23874,12 +24529,12 @@
         <v>2472</v>
       </c>
     </row>
-    <row r="51" spans="1:43">
+    <row r="51" spans="1:43" ht="15">
       <c r="A51" s="7" t="s">
         <v>3260</v>
       </c>
     </row>
-    <row r="52" spans="1:43">
+    <row r="52" spans="1:43" ht="15">
       <c r="A52" s="7" t="s">
         <v>3261</v>
       </c>
@@ -23890,7 +24545,7 @@
         <v>2473</v>
       </c>
     </row>
-    <row r="53" spans="1:43">
+    <row r="53" spans="1:43" ht="15">
       <c r="A53" s="7" t="s">
         <v>3262</v>
       </c>
@@ -24255,7 +24910,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="89" spans="1:63">
+    <row r="89" spans="1:63" ht="15">
       <c r="AM89" s="16" t="s">
         <v>2537</v>
       </c>
@@ -24268,7 +24923,7 @@
       <c r="AT89" s="17"/>
       <c r="AU89" s="17"/>
     </row>
-    <row r="90" spans="1:63">
+    <row r="90" spans="1:63" ht="15">
       <c r="A90" s="16" t="s">
         <v>2492</v>
       </c>
@@ -24286,7 +24941,7 @@
         <v>2567</v>
       </c>
     </row>
-    <row r="91" spans="1:63">
+    <row r="91" spans="1:63" ht="15">
       <c r="A91" s="49" t="s">
         <v>3263</v>
       </c>
@@ -24300,7 +24955,7 @@
         <v>3271</v>
       </c>
     </row>
-    <row r="92" spans="1:63">
+    <row r="92" spans="1:63" ht="15">
       <c r="A92" s="8" t="s">
         <v>2493</v>
       </c>
@@ -24314,7 +24969,7 @@
         <v>3272</v>
       </c>
     </row>
-    <row r="93" spans="1:63">
+    <row r="93" spans="1:63" ht="15">
       <c r="A93" s="12"/>
       <c r="W93" s="10" t="s">
         <v>2518</v>
@@ -24326,7 +24981,7 @@
         <v>3273</v>
       </c>
     </row>
-    <row r="94" spans="1:63">
+    <row r="94" spans="1:63" ht="15">
       <c r="A94" s="7" t="s">
         <v>3264</v>
       </c>
@@ -24334,7 +24989,7 @@
         <v>2519</v>
       </c>
     </row>
-    <row r="95" spans="1:63">
+    <row r="95" spans="1:63" ht="15">
       <c r="A95" s="7" t="s">
         <v>3265</v>
       </c>
@@ -24348,7 +25003,7 @@
         <v>2568</v>
       </c>
     </row>
-    <row r="96" spans="1:63">
+    <row r="96" spans="1:63" ht="15">
       <c r="A96" s="7" t="s">
         <v>3266</v>
       </c>
@@ -24362,7 +25017,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="97" spans="1:63">
+    <row r="97" spans="1:63" ht="15">
       <c r="A97" s="7" t="s">
         <v>3267</v>
       </c>
@@ -24892,7 +25547,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="144" spans="1:63">
+    <row r="144" spans="1:63" ht="15">
       <c r="A144" s="16" t="s">
         <v>2595</v>
       </c>
@@ -24902,7 +25557,7 @@
       <c r="E144" s="17"/>
       <c r="F144" s="17"/>
     </row>
-    <row r="145" spans="1:50">
+    <row r="145" spans="1:50" ht="15">
       <c r="A145" s="52" t="s">
         <v>3283</v>
       </c>
@@ -24910,7 +25565,7 @@
         <v>2612</v>
       </c>
     </row>
-    <row r="146" spans="1:50">
+    <row r="146" spans="1:50" ht="15">
       <c r="A146" s="8" t="s">
         <v>2596</v>
       </c>
@@ -25373,13 +26028,13 @@
         <v>46</v>
       </c>
     </row>
-    <row r="203" spans="1:79" ht="14.4" thickBot="1"/>
-    <row r="204" spans="1:79" s="14" customFormat="1" ht="14.4" thickBot="1">
+    <row r="203" spans="1:79" ht="15" thickBot="1"/>
+    <row r="204" spans="1:79" s="14" customFormat="1" ht="15.75" thickBot="1">
       <c r="A204" s="13" t="s">
         <v>2667</v>
       </c>
     </row>
-    <row r="205" spans="1:79">
+    <row r="205" spans="1:79" ht="15">
       <c r="A205" s="16" t="s">
         <v>2668</v>
       </c>
@@ -25420,7 +26075,7 @@
       <c r="BZ205" s="17"/>
       <c r="CA205" s="17"/>
     </row>
-    <row r="206" spans="1:79">
+    <row r="206" spans="1:79" ht="15">
       <c r="A206" s="18" t="s">
         <v>2669</v>
       </c>
@@ -25461,7 +26116,7 @@
         <v>1521</v>
       </c>
     </row>
-    <row r="208" spans="1:79">
+    <row r="208" spans="1:79" ht="15">
       <c r="A208" s="8" t="s">
         <v>2670</v>
       </c>
@@ -25472,7 +26127,7 @@
         <v>1522</v>
       </c>
     </row>
-    <row r="209" spans="1:83">
+    <row r="209" spans="1:83" ht="15">
       <c r="A209" s="10" t="s">
         <v>2671</v>
       </c>
@@ -25867,7 +26522,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="237" spans="1:85">
+    <row r="237" spans="1:85" ht="15">
       <c r="A237" s="8" t="s">
         <v>2693</v>
       </c>
@@ -25876,7 +26531,7 @@
       </c>
       <c r="BS237" s="11"/>
     </row>
-    <row r="238" spans="1:85">
+    <row r="238" spans="1:85" ht="15">
       <c r="A238" s="10" t="s">
         <v>2694</v>
       </c>
@@ -26101,7 +26756,7 @@
       </c>
       <c r="AV253" s="11"/>
     </row>
-    <row r="254" spans="1:71">
+    <row r="254" spans="1:71" ht="15">
       <c r="A254" s="10" t="s">
         <v>46</v>
       </c>
@@ -26128,7 +26783,7 @@
         <v>1552</v>
       </c>
     </row>
-    <row r="256" spans="1:71">
+    <row r="256" spans="1:71" ht="15">
       <c r="A256" s="10" t="s">
         <v>2703</v>
       </c>
@@ -26289,7 +26944,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="267" spans="1:71">
+    <row r="267" spans="1:71" ht="15">
       <c r="A267" s="8" t="s">
         <v>2710</v>
       </c>
@@ -26586,7 +27241,7 @@
         <v>1488</v>
       </c>
     </row>
-    <row r="295" spans="1:71">
+    <row r="295" spans="1:71" ht="15">
       <c r="A295" s="10" t="s">
         <v>2731</v>
       </c>
@@ -26757,7 +27412,7 @@
         <v>1585</v>
       </c>
     </row>
-    <row r="311" spans="1:71">
+    <row r="311" spans="1:71" ht="15">
       <c r="A311" s="10" t="s">
         <v>294</v>
       </c>
@@ -26773,7 +27428,7 @@
         <v>1586</v>
       </c>
     </row>
-    <row r="312" spans="1:71">
+    <row r="312" spans="1:71" ht="15">
       <c r="A312" s="10" t="s">
         <v>2743</v>
       </c>
@@ -27051,13 +27706,13 @@
         <v>1518</v>
       </c>
     </row>
-    <row r="338" spans="1:67" ht="14.4" thickBot="1"/>
-    <row r="339" spans="1:67" s="14" customFormat="1" ht="14.4" thickBot="1">
+    <row r="338" spans="1:67" ht="15" thickBot="1"/>
+    <row r="339" spans="1:67" s="14" customFormat="1" ht="15.75" thickBot="1">
       <c r="A339" s="13" t="s">
         <v>1593</v>
       </c>
     </row>
-    <row r="340" spans="1:67">
+    <row r="340" spans="1:67" ht="15">
       <c r="A340" s="16" t="s">
         <v>1594</v>
       </c>
@@ -27124,7 +27779,7 @@
         <v>1666</v>
       </c>
     </row>
-    <row r="342" spans="1:67">
+    <row r="342" spans="1:67" ht="15">
       <c r="A342" s="10" t="s">
         <v>1596</v>
       </c>
@@ -27216,7 +27871,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="349" spans="1:67">
+    <row r="349" spans="1:67" ht="15">
       <c r="A349" s="11"/>
       <c r="W349" s="42" t="s">
         <v>1631</v>
@@ -27608,13 +28263,13 @@
         <v>46</v>
       </c>
     </row>
-    <row r="384" spans="1:57" ht="14.4" thickBot="1"/>
-    <row r="385" spans="1:26" s="14" customFormat="1" ht="14.4" thickBot="1">
+    <row r="384" spans="1:57" ht="15" thickBot="1"/>
+    <row r="385" spans="1:26" s="14" customFormat="1" ht="15.75" thickBot="1">
       <c r="A385" s="13" t="s">
         <v>1686</v>
       </c>
     </row>
-    <row r="386" spans="1:26">
+    <row r="386" spans="1:26" ht="15">
       <c r="A386" s="8" t="s">
         <v>1687</v>
       </c>
@@ -28293,7 +28948,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="478" spans="1:65">
+    <row r="478" spans="1:65" ht="15">
       <c r="A478" s="8" t="s">
         <v>1796</v>
       </c>
@@ -30294,17 +30949,17 @@
         <v>719</v>
       </c>
     </row>
-    <row r="669" spans="1:65" ht="14.4" thickBot="1">
+    <row r="669" spans="1:65" ht="15" thickBot="1">
       <c r="A669" s="11" t="s">
         <v>3281</v>
       </c>
     </row>
-    <row r="670" spans="1:65" s="14" customFormat="1" ht="14.4" thickBot="1">
+    <row r="670" spans="1:65" s="14" customFormat="1" ht="15.75" thickBot="1">
       <c r="A670" s="55" t="s">
         <v>3279</v>
       </c>
     </row>
-    <row r="671" spans="1:65">
+    <row r="671" spans="1:65" ht="15">
       <c r="A671" s="51" t="s">
         <v>3280</v>
       </c>
@@ -31059,17 +31714,17 @@
         <v>2262</v>
       </c>
     </row>
-    <row r="783" spans="1:32" ht="14.4" thickBot="1">
+    <row r="783" spans="1:32" ht="15" thickBot="1">
       <c r="AF783" s="10" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="784" spans="1:32" s="14" customFormat="1" ht="14.4" thickBot="1">
+    <row r="784" spans="1:32" s="14" customFormat="1" ht="15.75" thickBot="1">
       <c r="A784" s="13" t="s">
         <v>2263</v>
       </c>
     </row>
-    <row r="785" spans="1:51">
+    <row r="785" spans="1:51" ht="15">
       <c r="A785" s="16" t="s">
         <v>2264</v>
       </c>
@@ -31093,7 +31748,7 @@
         <v>2917</v>
       </c>
     </row>
-    <row r="786" spans="1:51">
+    <row r="786" spans="1:51" ht="15">
       <c r="A786" s="10" t="s">
         <v>2265</v>
       </c>
@@ -31929,7 +32584,7 @@
         <v>2974</v>
       </c>
     </row>
-    <row r="860" spans="1:51">
+    <row r="860" spans="1:51" ht="15">
       <c r="A860" s="8" t="s">
         <v>2320</v>
       </c>
@@ -32091,7 +32746,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="876" spans="1:51">
+    <row r="876" spans="1:51" ht="15">
       <c r="A876" s="10" t="s">
         <v>2331</v>
       </c>
@@ -32750,17 +33405,17 @@
         <v>3039</v>
       </c>
     </row>
-    <row r="957" spans="1:54" ht="14.4" thickBot="1">
+    <row r="957" spans="1:54" ht="15" thickBot="1">
       <c r="AY957" s="10" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="958" spans="1:54" s="14" customFormat="1" ht="14.4" thickBot="1">
+    <row r="958" spans="1:54" s="14" customFormat="1" ht="15.75" thickBot="1">
       <c r="A958" s="13" t="s">
         <v>3040</v>
       </c>
     </row>
-    <row r="959" spans="1:54">
+    <row r="959" spans="1:54" ht="15">
       <c r="A959" s="8" t="s">
         <v>3041</v>
       </c>
@@ -34032,18 +34687,18 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:BO608"/>
-  <sheetFormatPr defaultColWidth="3.09765625" defaultRowHeight="13.8"/>
+  <dimension ref="A1:BS608"/>
+  <sheetFormatPr defaultColWidth="3.125" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="16384" width="3.09765625" style="9"/>
+    <col min="1" max="16384" width="3.125" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:56" s="14" customFormat="1" ht="14.4" thickBot="1">
+    <row r="1" spans="1:56" s="14" customFormat="1" ht="15.75" thickBot="1">
       <c r="A1" s="13" t="s">
         <v>3649</v>
       </c>
     </row>
-    <row r="2" spans="1:56">
+    <row r="2" spans="1:56" ht="15">
       <c r="A2" s="16" t="s">
         <v>3650</v>
       </c>
@@ -34076,9 +34731,9 @@
       <c r="BA2" s="17"/>
       <c r="BB2" s="17"/>
     </row>
-    <row r="3" spans="1:56">
+    <row r="3" spans="1:56" ht="15">
       <c r="A3" s="7" t="s">
-        <v>4097</v>
+        <v>4094</v>
       </c>
       <c r="AF3" s="10" t="s">
         <v>3657</v>
@@ -34090,9 +34745,9 @@
       <c r="AT3" s="18"/>
       <c r="AU3" s="18"/>
     </row>
-    <row r="4" spans="1:56">
+    <row r="4" spans="1:56" ht="15">
       <c r="A4" s="7" t="s">
-        <v>4098</v>
+        <v>4095</v>
       </c>
       <c r="AF4" s="10" t="s">
         <v>3468</v>
@@ -34130,9 +34785,9 @@
       <c r="AT6" s="18"/>
       <c r="AU6" s="18"/>
     </row>
-    <row r="7" spans="1:56">
+    <row r="7" spans="1:56" ht="15">
       <c r="A7" s="7" t="s">
-        <v>4099</v>
+        <v>4096</v>
       </c>
       <c r="AF7" s="10" t="s">
         <v>3659</v>
@@ -34178,13 +34833,13 @@
         <v>46</v>
       </c>
     </row>
-    <row r="13" spans="1:56" ht="14.4" thickBot="1"/>
-    <row r="14" spans="1:56" s="14" customFormat="1" ht="14.4" thickBot="1">
+    <row r="13" spans="1:56" ht="15" thickBot="1"/>
+    <row r="14" spans="1:56" s="14" customFormat="1" ht="15.75" thickBot="1">
       <c r="A14" s="13" t="s">
         <v>3671</v>
       </c>
     </row>
-    <row r="15" spans="1:56">
+    <row r="15" spans="1:56" ht="15">
       <c r="A15" s="16" t="s">
         <v>3672</v>
       </c>
@@ -34214,9 +34869,9 @@
       <c r="BC15" s="17"/>
       <c r="BD15" s="17"/>
     </row>
-    <row r="16" spans="1:56">
+    <row r="16" spans="1:56" ht="15">
       <c r="A16" s="7" t="s">
-        <v>4100</v>
+        <v>4097</v>
       </c>
       <c r="X16" s="10" t="s">
         <v>3693</v>
@@ -34225,9 +34880,9 @@
         <v>3704</v>
       </c>
     </row>
-    <row r="17" spans="1:47">
+    <row r="17" spans="1:47" ht="15">
       <c r="A17" s="7" t="s">
-        <v>4101</v>
+        <v>4098</v>
       </c>
       <c r="X17" s="10" t="s">
         <v>3694</v>
@@ -34236,9 +34891,9 @@
         <v>66</v>
       </c>
     </row>
-    <row r="18" spans="1:47">
+    <row r="18" spans="1:47" ht="15">
       <c r="A18" s="7" t="s">
-        <v>4102</v>
+        <v>4099</v>
       </c>
       <c r="X18" s="10" t="s">
         <v>3695</v>
@@ -34255,7 +34910,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="20" spans="1:47">
+    <row r="20" spans="1:47" ht="15">
       <c r="A20" s="16" t="s">
         <v>3673</v>
       </c>
@@ -34445,13 +35100,13 @@
         <v>3691</v>
       </c>
     </row>
-    <row r="46" spans="1:47" ht="14.4" thickBot="1"/>
-    <row r="47" spans="1:47" s="14" customFormat="1" ht="14.4" thickBot="1">
+    <row r="46" spans="1:47" ht="15" thickBot="1"/>
+    <row r="47" spans="1:47" s="14" customFormat="1" ht="15.75" thickBot="1">
       <c r="A47" s="13" t="s">
         <v>3719</v>
       </c>
     </row>
-    <row r="48" spans="1:47">
+    <row r="48" spans="1:47" ht="15">
       <c r="A48" s="8" t="s">
         <v>3720</v>
       </c>
@@ -34638,17 +35293,17 @@
         <v>3758</v>
       </c>
     </row>
-    <row r="73" spans="1:40" ht="14.4" thickBot="1">
+    <row r="73" spans="1:40" ht="15" thickBot="1">
       <c r="Q73" s="10" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="74" spans="1:40" s="14" customFormat="1" ht="14.4" thickBot="1">
+    <row r="74" spans="1:40" s="14" customFormat="1" ht="15.75" thickBot="1">
       <c r="A74" s="13" t="s">
         <v>3759</v>
       </c>
     </row>
-    <row r="75" spans="1:40">
+    <row r="75" spans="1:40" ht="15">
       <c r="A75" s="16" t="s">
         <v>3760</v>
       </c>
@@ -34975,13 +35630,13 @@
         <v>46</v>
       </c>
     </row>
-    <row r="108" spans="1:50" ht="14.4" thickBot="1"/>
-    <row r="109" spans="1:50" s="14" customFormat="1" ht="14.4" thickBot="1">
+    <row r="108" spans="1:50" ht="15" thickBot="1"/>
+    <row r="109" spans="1:50" s="14" customFormat="1" ht="15.75" thickBot="1">
       <c r="A109" s="13" t="s">
         <v>3818</v>
       </c>
     </row>
-    <row r="110" spans="1:50">
+    <row r="110" spans="1:50" ht="15">
       <c r="A110" s="16" t="s">
         <v>3819</v>
       </c>
@@ -35236,7 +35891,7 @@
     </row>
     <row r="132" spans="1:46">
       <c r="A132" s="10" t="s">
-        <v>4103</v>
+        <v>4100</v>
       </c>
       <c r="W132" s="15" t="s">
         <v>3852</v>
@@ -35453,24 +36108,24 @@
         <v>171</v>
       </c>
     </row>
-    <row r="162" spans="1:46" ht="14.4" thickBot="1">
+    <row r="162" spans="1:46" ht="15" thickBot="1">
       <c r="AT162" s="10" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="163" spans="1:46" s="58" customFormat="1" ht="14.4" thickBot="1">
+    <row r="163" spans="1:46" s="58" customFormat="1" ht="15.75" thickBot="1">
       <c r="A163" s="57" t="s">
         <v>3893</v>
       </c>
     </row>
-    <row r="164" spans="1:46" s="60" customFormat="1" ht="14.4" thickBot="1">
+    <row r="164" spans="1:46" s="60" customFormat="1" ht="15.75" thickBot="1">
       <c r="A164" s="59" t="s">
+        <v>4113</v>
+      </c>
+    </row>
+    <row r="165" spans="1:46" ht="15">
+      <c r="A165" s="43" t="s">
         <v>3894</v>
-      </c>
-    </row>
-    <row r="165" spans="1:46">
-      <c r="A165" s="43" t="s">
-        <v>3895</v>
       </c>
       <c r="B165" s="20"/>
       <c r="C165" s="20"/>
@@ -35481,15 +36136,15 @@
     </row>
     <row r="166" spans="1:46">
       <c r="A166" s="15" t="s">
-        <v>3896</v>
+        <v>3895</v>
       </c>
     </row>
     <row r="167" spans="1:46">
       <c r="A167" s="10" t="s">
-        <v>3897</v>
+        <v>3896</v>
       </c>
       <c r="W167" s="15" t="s">
-        <v>3944</v>
+        <v>3943</v>
       </c>
     </row>
     <row r="168" spans="1:46">
@@ -35497,7 +36152,7 @@
         <v>3839</v>
       </c>
       <c r="W168" s="10" t="s">
-        <v>3945</v>
+        <v>3944</v>
       </c>
     </row>
     <row r="169" spans="1:46">
@@ -35505,12 +36160,12 @@
         <v>3443</v>
       </c>
       <c r="W169" s="10" t="s">
-        <v>3946</v>
+        <v>3945</v>
       </c>
     </row>
     <row r="170" spans="1:46">
       <c r="A170" s="10" t="s">
-        <v>3898</v>
+        <v>3897</v>
       </c>
       <c r="W170" s="11"/>
     </row>
@@ -35518,151 +36173,223 @@
       <c r="A171" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="W171" s="9" t="s">
+      <c r="W171" s="72" t="s">
         <v>53</v>
       </c>
+      <c r="X171" s="73"/>
+      <c r="Y171" s="73"/>
+      <c r="Z171" s="73"/>
+      <c r="AA171" s="73"/>
+      <c r="AB171" s="73"/>
+      <c r="AC171" s="73"/>
+      <c r="AD171" s="73"/>
+      <c r="AE171" s="73"/>
+      <c r="AF171" s="74"/>
     </row>
     <row r="172" spans="1:46">
       <c r="A172" s="15" t="s">
-        <v>3899</v>
-      </c>
-      <c r="W172" s="9" t="s">
-        <v>4105</v>
-      </c>
+        <v>3898</v>
+      </c>
+      <c r="W172" s="75" t="s">
+        <v>4102</v>
+      </c>
+      <c r="X172" s="76"/>
+      <c r="Y172" s="76"/>
+      <c r="Z172" s="76"/>
+      <c r="AA172" s="76"/>
+      <c r="AB172" s="76"/>
+      <c r="AC172" s="76"/>
+      <c r="AD172" s="76"/>
+      <c r="AE172" s="76"/>
+      <c r="AF172" s="77"/>
     </row>
     <row r="173" spans="1:46">
       <c r="A173" s="10" t="s">
-        <v>3900</v>
-      </c>
-      <c r="W173" s="9" t="s">
-        <v>4106</v>
-      </c>
+        <v>3899</v>
+      </c>
+      <c r="W173" s="75" t="s">
+        <v>4103</v>
+      </c>
+      <c r="X173" s="76"/>
+      <c r="Y173" s="76"/>
+      <c r="Z173" s="76"/>
+      <c r="AA173" s="76"/>
+      <c r="AB173" s="76"/>
+      <c r="AC173" s="76"/>
+      <c r="AD173" s="76"/>
+      <c r="AE173" s="76"/>
+      <c r="AF173" s="77"/>
     </row>
     <row r="174" spans="1:46">
       <c r="A174" s="10" t="s">
-        <v>3901</v>
-      </c>
-      <c r="W174" s="9" t="s">
-        <v>4107</v>
-      </c>
+        <v>3900</v>
+      </c>
+      <c r="W174" s="75" t="s">
+        <v>4104</v>
+      </c>
+      <c r="X174" s="76"/>
+      <c r="Y174" s="76"/>
+      <c r="Z174" s="76"/>
+      <c r="AA174" s="76"/>
+      <c r="AB174" s="76"/>
+      <c r="AC174" s="76"/>
+      <c r="AD174" s="76"/>
+      <c r="AE174" s="76"/>
+      <c r="AF174" s="77"/>
     </row>
     <row r="175" spans="1:46">
       <c r="A175" s="10" t="s">
-        <v>3902</v>
-      </c>
-      <c r="W175" s="9" t="s">
-        <v>4108</v>
-      </c>
+        <v>3901</v>
+      </c>
+      <c r="W175" s="75" t="s">
+        <v>4105</v>
+      </c>
+      <c r="X175" s="76"/>
+      <c r="Y175" s="76"/>
+      <c r="Z175" s="76"/>
+      <c r="AA175" s="76"/>
+      <c r="AB175" s="76"/>
+      <c r="AC175" s="76"/>
+      <c r="AD175" s="76"/>
+      <c r="AE175" s="76"/>
+      <c r="AF175" s="77"/>
     </row>
     <row r="176" spans="1:46">
       <c r="A176" s="10" t="s">
+        <v>3902</v>
+      </c>
+      <c r="W176" s="75" t="s">
+        <v>4106</v>
+      </c>
+      <c r="X176" s="76"/>
+      <c r="Y176" s="76"/>
+      <c r="Z176" s="76"/>
+      <c r="AA176" s="76"/>
+      <c r="AB176" s="76"/>
+      <c r="AC176" s="76"/>
+      <c r="AD176" s="76"/>
+      <c r="AE176" s="76"/>
+      <c r="AF176" s="77"/>
+    </row>
+    <row r="177" spans="1:32">
+      <c r="A177" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="W177" s="75" t="s">
+        <v>4107</v>
+      </c>
+      <c r="X177" s="76"/>
+      <c r="Y177" s="76"/>
+      <c r="Z177" s="76"/>
+      <c r="AA177" s="76"/>
+      <c r="AB177" s="76"/>
+      <c r="AC177" s="76"/>
+      <c r="AD177" s="76"/>
+      <c r="AE177" s="76"/>
+      <c r="AF177" s="77"/>
+    </row>
+    <row r="178" spans="1:32">
+      <c r="A178" s="15" t="s">
         <v>3903</v>
       </c>
-      <c r="W176" s="9" t="s">
-        <v>4109</v>
-      </c>
-    </row>
-    <row r="177" spans="1:23">
-      <c r="A177" s="10" t="s">
-        <v>101</v>
-      </c>
-      <c r="W177" s="9" t="s">
-        <v>4110</v>
-      </c>
-    </row>
-    <row r="178" spans="1:23">
-      <c r="A178" s="15" t="s">
+      <c r="W178" s="78" t="s">
+        <v>3946</v>
+      </c>
+      <c r="X178" s="79"/>
+      <c r="Y178" s="79"/>
+      <c r="Z178" s="79"/>
+      <c r="AA178" s="79"/>
+      <c r="AB178" s="79"/>
+      <c r="AC178" s="79"/>
+      <c r="AD178" s="79"/>
+      <c r="AE178" s="79"/>
+      <c r="AF178" s="80"/>
+    </row>
+    <row r="179" spans="1:32">
+      <c r="A179" s="10" t="s">
         <v>3904</v>
       </c>
-      <c r="W178" s="9" t="s">
+      <c r="W179" s="11"/>
+    </row>
+    <row r="180" spans="1:32">
+      <c r="A180" s="10" t="s">
+        <v>3905</v>
+      </c>
+      <c r="W180" s="10" t="s">
         <v>3947</v>
       </c>
     </row>
-    <row r="179" spans="1:23">
-      <c r="A179" s="10" t="s">
-        <v>3905</v>
-      </c>
-      <c r="W179" s="11"/>
-    </row>
-    <row r="180" spans="1:23">
-      <c r="A180" s="10" t="s">
+    <row r="181" spans="1:32">
+      <c r="A181" s="10" t="s">
         <v>3906</v>
       </c>
-      <c r="W180" s="10" t="s">
+      <c r="W181" s="10" t="s">
         <v>3948</v>
       </c>
     </row>
-    <row r="181" spans="1:23">
-      <c r="A181" s="10" t="s">
+    <row r="182" spans="1:32">
+      <c r="A182" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="W182" s="10" t="s">
+        <v>3949</v>
+      </c>
+    </row>
+    <row r="183" spans="1:32">
+      <c r="A183" s="15" t="s">
         <v>3907</v>
       </c>
-      <c r="W181" s="10" t="s">
-        <v>3949</v>
-      </c>
-    </row>
-    <row r="182" spans="1:23">
-      <c r="A182" s="10" t="s">
-        <v>101</v>
-      </c>
-      <c r="W182" s="10" t="s">
+      <c r="W183" s="10" t="s">
         <v>3950</v>
       </c>
     </row>
-    <row r="183" spans="1:23">
-      <c r="A183" s="15" t="s">
+    <row r="184" spans="1:32">
+      <c r="A184" s="10" t="s">
         <v>3908</v>
-      </c>
-      <c r="W183" s="10" t="s">
-        <v>3951</v>
-      </c>
-    </row>
-    <row r="184" spans="1:23">
-      <c r="A184" s="10" t="s">
-        <v>3909</v>
       </c>
       <c r="W184" s="10" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="185" spans="1:23">
+    <row r="185" spans="1:32">
       <c r="A185" s="10" t="s">
+        <v>3909</v>
+      </c>
+      <c r="W185" s="10" t="s">
+        <v>3951</v>
+      </c>
+    </row>
+    <row r="186" spans="1:32">
+      <c r="A186" s="10" t="s">
         <v>3910</v>
-      </c>
-      <c r="W185" s="10" t="s">
-        <v>3952</v>
-      </c>
-    </row>
-    <row r="186" spans="1:23">
-      <c r="A186" s="10" t="s">
-        <v>3911</v>
       </c>
       <c r="W186" s="10" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="187" spans="1:23">
+    <row r="187" spans="1:32">
       <c r="A187" s="10" t="s">
         <v>46</v>
       </c>
       <c r="W187" s="11"/>
     </row>
-    <row r="188" spans="1:23">
+    <row r="188" spans="1:32">
       <c r="A188" s="11"/>
       <c r="W188" s="10" t="s">
+        <v>3952</v>
+      </c>
+    </row>
+    <row r="189" spans="1:32">
+      <c r="A189" s="15" t="s">
+        <v>3911</v>
+      </c>
+      <c r="W189" s="10" t="s">
         <v>3953</v>
       </c>
     </row>
-    <row r="189" spans="1:23">
-      <c r="A189" s="15" t="s">
+    <row r="190" spans="1:32" ht="15">
+      <c r="A190" s="64" t="s">
         <v>3912</v>
-      </c>
-      <c r="W189" s="10" t="s">
-        <v>3954</v>
-      </c>
-    </row>
-    <row r="190" spans="1:23">
-      <c r="A190" s="64" t="s">
-        <v>3913</v>
       </c>
       <c r="B190" s="65"/>
       <c r="C190" s="65"/>
@@ -35682,12 +36409,12 @@
       <c r="Q190" s="65"/>
       <c r="R190" s="65"/>
       <c r="W190" s="10" t="s">
-        <v>3955</v>
-      </c>
-    </row>
-    <row r="191" spans="1:23">
+        <v>3954</v>
+      </c>
+    </row>
+    <row r="191" spans="1:32">
       <c r="A191" s="66" t="s">
-        <v>3914</v>
+        <v>3913</v>
       </c>
       <c r="B191" s="65"/>
       <c r="C191" s="65"/>
@@ -35707,12 +36434,12 @@
       <c r="Q191" s="65"/>
       <c r="R191" s="65"/>
       <c r="W191" s="10" t="s">
-        <v>3956</v>
-      </c>
-    </row>
-    <row r="192" spans="1:23">
+        <v>3955</v>
+      </c>
+    </row>
+    <row r="192" spans="1:32">
       <c r="A192" s="66" t="s">
-        <v>3915</v>
+        <v>3914</v>
       </c>
       <c r="B192" s="65"/>
       <c r="C192" s="65"/>
@@ -35732,7 +36459,7 @@
       <c r="Q192" s="65"/>
       <c r="R192" s="65"/>
       <c r="W192" s="10" t="s">
-        <v>3957</v>
+        <v>3956</v>
       </c>
     </row>
     <row r="193" spans="1:23">
@@ -35763,12 +36490,12 @@
     <row r="194" spans="1:23">
       <c r="A194" s="11"/>
       <c r="W194" s="10" t="s">
-        <v>3950</v>
-      </c>
-    </row>
-    <row r="195" spans="1:23">
+        <v>3949</v>
+      </c>
+    </row>
+    <row r="195" spans="1:23" ht="15">
       <c r="A195" s="67" t="s">
-        <v>3916</v>
+        <v>3915</v>
       </c>
       <c r="B195" s="68"/>
       <c r="C195" s="68"/>
@@ -35788,12 +36515,12 @@
       <c r="Q195" s="68"/>
       <c r="R195" s="68"/>
       <c r="W195" s="10" t="s">
-        <v>3958</v>
+        <v>3957</v>
       </c>
     </row>
     <row r="196" spans="1:23">
       <c r="A196" s="69" t="s">
-        <v>3917</v>
+        <v>3916</v>
       </c>
       <c r="B196" s="68"/>
       <c r="C196" s="68"/>
@@ -35818,7 +36545,7 @@
     </row>
     <row r="197" spans="1:23">
       <c r="A197" s="69" t="s">
-        <v>3918</v>
+        <v>3917</v>
       </c>
       <c r="B197" s="68"/>
       <c r="C197" s="68"/>
@@ -35863,7 +36590,7 @@
       <c r="Q198" s="68"/>
       <c r="R198" s="68"/>
       <c r="W198" s="10" t="s">
-        <v>3959</v>
+        <v>3958</v>
       </c>
     </row>
     <row r="199" spans="1:23">
@@ -35888,7 +36615,7 @@
       <c r="Q199" s="68"/>
       <c r="R199" s="68"/>
       <c r="W199" s="10" t="s">
-        <v>3960</v>
+        <v>3959</v>
       </c>
     </row>
     <row r="200" spans="1:23">
@@ -35899,15 +36626,15 @@
     </row>
     <row r="201" spans="1:23">
       <c r="A201" s="15" t="s">
-        <v>3919</v>
+        <v>3918</v>
       </c>
       <c r="W201" s="10" t="s">
-        <v>3961</v>
+        <v>3960</v>
       </c>
     </row>
     <row r="202" spans="1:23">
       <c r="A202" s="10" t="s">
-        <v>3920</v>
+        <v>3919</v>
       </c>
       <c r="W202" s="10" t="s">
         <v>46</v>
@@ -35915,12 +36642,12 @@
     </row>
     <row r="203" spans="1:23">
       <c r="A203" s="10" t="s">
-        <v>3921</v>
+        <v>3920</v>
       </c>
     </row>
     <row r="204" spans="1:23">
       <c r="A204" s="10" t="s">
-        <v>3922</v>
+        <v>3921</v>
       </c>
     </row>
     <row r="205" spans="1:23">
@@ -35933,84 +36660,114 @@
     </row>
     <row r="207" spans="1:23">
       <c r="A207" s="15" t="s">
-        <v>3923</v>
+        <v>3922</v>
       </c>
     </row>
     <row r="208" spans="1:23">
       <c r="A208" s="10" t="s">
+        <v>3923</v>
+      </c>
+    </row>
+    <row r="209" spans="1:71">
+      <c r="A209" s="10" t="s">
         <v>3924</v>
       </c>
     </row>
-    <row r="209" spans="1:1">
-      <c r="A209" s="10" t="s">
+    <row r="210" spans="1:71">
+      <c r="A210" s="10" t="s">
         <v>3925</v>
       </c>
     </row>
-    <row r="210" spans="1:1">
-      <c r="A210" s="10" t="s">
-        <v>3926</v>
-      </c>
-    </row>
-    <row r="211" spans="1:1">
+    <row r="211" spans="1:71">
       <c r="A211" s="10" t="s">
         <v>343</v>
       </c>
     </row>
-    <row r="212" spans="1:1">
+    <row r="212" spans="1:71" ht="20.25">
       <c r="A212" s="10" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="213" spans="1:1">
+      <c r="AB212" s="71" t="s">
+        <v>4108</v>
+      </c>
+      <c r="BJ212" s="83" t="s">
+        <v>4121</v>
+      </c>
+      <c r="BK212" s="84"/>
+      <c r="BL212" s="84"/>
+      <c r="BM212" s="84"/>
+      <c r="BN212" s="84"/>
+      <c r="BO212" s="84"/>
+      <c r="BP212" s="85"/>
+    </row>
+    <row r="213" spans="1:71">
       <c r="A213" s="11"/>
-    </row>
-    <row r="214" spans="1:1">
+      <c r="AC213" s="9" t="s">
+        <v>4109</v>
+      </c>
+    </row>
+    <row r="214" spans="1:71" ht="15">
       <c r="A214" s="15" t="s">
+        <v>3926</v>
+      </c>
+      <c r="BJ214" s="86" t="s">
+        <v>4125</v>
+      </c>
+      <c r="BK214" s="87"/>
+      <c r="BL214" s="87"/>
+      <c r="BM214" s="87"/>
+      <c r="BN214" s="87"/>
+      <c r="BO214" s="87"/>
+      <c r="BP214" s="87"/>
+      <c r="BQ214" s="87"/>
+      <c r="BR214" s="88"/>
+      <c r="BS214" s="85"/>
+    </row>
+    <row r="215" spans="1:71" ht="20.25">
+      <c r="A215" s="10" t="s">
         <v>3927</v>
       </c>
-    </row>
-    <row r="215" spans="1:1">
-      <c r="A215" s="10" t="s">
-        <v>3928</v>
-      </c>
-    </row>
-    <row r="216" spans="1:1">
+      <c r="AB215" s="71" t="s">
+        <v>4110</v>
+      </c>
+    </row>
+    <row r="216" spans="1:71">
       <c r="A216" s="10" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="217" spans="1:1">
+    <row r="217" spans="1:71">
       <c r="A217" s="10" t="s">
+        <v>3928</v>
+      </c>
+    </row>
+    <row r="218" spans="1:71">
+      <c r="A218" s="10" t="s">
         <v>3929</v>
       </c>
     </row>
-    <row r="218" spans="1:1">
-      <c r="A218" s="10" t="s">
+    <row r="219" spans="1:71">
+      <c r="A219" s="10" t="s">
         <v>3930</v>
       </c>
     </row>
-    <row r="219" spans="1:1">
-      <c r="A219" s="10" t="s">
-        <v>3931</v>
-      </c>
-    </row>
-    <row r="220" spans="1:1">
+    <row r="220" spans="1:71">
       <c r="A220" s="10" t="s">
         <v>732</v>
       </c>
     </row>
-    <row r="221" spans="1:1">
+    <row r="221" spans="1:71">
       <c r="A221" s="11"/>
     </row>
-    <row r="222" spans="1:1">
+    <row r="222" spans="1:71">
       <c r="A222" s="10" t="s">
-        <v>3932</v>
-      </c>
-    </row>
-    <row r="223" spans="1:1">
+        <v>3931</v>
+      </c>
+    </row>
+    <row r="223" spans="1:71">
       <c r="A223" s="11"/>
     </row>
-    <row r="224" spans="1:1">
+    <row r="224" spans="1:71">
       <c r="A224" s="15" t="s">
         <v>287</v>
       </c>
@@ -36022,25 +36779,25 @@
     </row>
     <row r="226" spans="1:20">
       <c r="A226" s="10" t="s">
-        <v>3933</v>
+        <v>3932</v>
       </c>
     </row>
     <row r="227" spans="1:20">
       <c r="A227" s="10" t="s">
-        <v>3934</v>
-      </c>
-    </row>
-    <row r="228" spans="1:20" ht="14.4" thickBot="1">
+        <v>3933</v>
+      </c>
+    </row>
+    <row r="228" spans="1:20" ht="15" thickBot="1">
       <c r="A228" s="10" t="s">
         <v>282</v>
       </c>
     </row>
-    <row r="229" spans="1:20" ht="14.4" thickBot="1">
+    <row r="229" spans="1:20" ht="15.75" thickBot="1">
       <c r="A229" s="10" t="s">
-        <v>3935</v>
+        <v>3934</v>
       </c>
       <c r="Q229" s="63" t="s">
-        <v>4104</v>
+        <v>4101</v>
       </c>
       <c r="R229" s="61"/>
       <c r="S229" s="62"/>
@@ -36048,12 +36805,12 @@
     </row>
     <row r="230" spans="1:20">
       <c r="A230" s="10" t="s">
-        <v>3936</v>
+        <v>3935</v>
       </c>
     </row>
     <row r="231" spans="1:20">
       <c r="A231" s="10" t="s">
-        <v>3937</v>
+        <v>3936</v>
       </c>
     </row>
     <row r="232" spans="1:20">
@@ -36076,52 +36833,72 @@
     </row>
     <row r="236" spans="1:20">
       <c r="A236" s="15" t="s">
-        <v>3938</v>
+        <v>3937</v>
       </c>
     </row>
     <row r="237" spans="1:20">
       <c r="A237" s="10" t="s">
-        <v>3939</v>
+        <v>3938</v>
       </c>
     </row>
     <row r="238" spans="1:20">
       <c r="A238" s="10" t="s">
-        <v>3940</v>
+        <v>3939</v>
       </c>
     </row>
     <row r="239" spans="1:20">
       <c r="A239" s="10" t="s">
-        <v>3941</v>
+        <v>3940</v>
       </c>
     </row>
     <row r="240" spans="1:20">
       <c r="A240" s="10" t="s">
-        <v>3942</v>
-      </c>
-    </row>
-    <row r="241" spans="1:28">
+        <v>3941</v>
+      </c>
+    </row>
+    <row r="241" spans="1:35" ht="15">
       <c r="A241" s="10" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="242" spans="1:28">
+      <c r="R241" s="81" t="s">
+        <v>4112</v>
+      </c>
+      <c r="S241" s="81"/>
+      <c r="T241" s="81"/>
+      <c r="U241" s="81"/>
+      <c r="V241" s="81"/>
+      <c r="W241" s="81"/>
+      <c r="X241" s="81"/>
+      <c r="Y241" s="81"/>
+      <c r="Z241" s="81"/>
+      <c r="AA241" s="81"/>
+      <c r="AB241" s="81"/>
+      <c r="AC241" s="81"/>
+      <c r="AD241" s="81"/>
+      <c r="AE241" s="81"/>
+      <c r="AF241" s="81"/>
+      <c r="AG241" s="81"/>
+      <c r="AH241" s="81"/>
+      <c r="AI241" s="82"/>
+    </row>
+    <row r="242" spans="1:35">
       <c r="A242" s="10" t="s">
-        <v>3943</v>
-      </c>
-    </row>
-    <row r="243" spans="1:28" ht="14.4" thickBot="1">
+        <v>3942</v>
+      </c>
+    </row>
+    <row r="243" spans="1:35" ht="15" thickBot="1">
       <c r="A243" s="10" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="244" spans="1:28" s="60" customFormat="1" ht="14.4" thickBot="1">
+    <row r="244" spans="1:35" s="60" customFormat="1" ht="15.75" thickBot="1">
       <c r="A244" s="59" t="s">
-        <v>3962</v>
-      </c>
-    </row>
-    <row r="245" spans="1:28">
+        <v>4111</v>
+      </c>
+    </row>
+    <row r="245" spans="1:35" ht="15">
       <c r="A245" s="43" t="s">
-        <v>3963</v>
+        <v>3961</v>
       </c>
       <c r="B245" s="20"/>
       <c r="C245" s="20"/>
@@ -36132,7 +36909,7 @@
       <c r="H245" s="20"/>
       <c r="I245" s="20"/>
       <c r="W245" s="43" t="s">
-        <v>4004</v>
+        <v>4002</v>
       </c>
       <c r="X245" s="20"/>
       <c r="Y245" s="20"/>
@@ -36140,135 +36917,147 @@
       <c r="AA245" s="20"/>
       <c r="AB245" s="20"/>
     </row>
-    <row r="246" spans="1:28">
+    <row r="246" spans="1:35">
       <c r="A246" s="15" t="s">
-        <v>3964</v>
+        <v>3962</v>
       </c>
       <c r="W246" s="10" t="s">
-        <v>4005</v>
-      </c>
-    </row>
-    <row r="247" spans="1:28">
+        <v>4003</v>
+      </c>
+    </row>
+    <row r="247" spans="1:35">
       <c r="A247" s="10" t="s">
-        <v>3965</v>
+        <v>3963</v>
       </c>
       <c r="W247" s="10" t="s">
-        <v>4006</v>
-      </c>
-    </row>
-    <row r="248" spans="1:28">
+        <v>4004</v>
+      </c>
+    </row>
+    <row r="248" spans="1:35">
       <c r="A248" s="15" t="s">
         <v>3839</v>
       </c>
       <c r="W248" s="10" t="s">
-        <v>4007</v>
-      </c>
-    </row>
-    <row r="249" spans="1:28">
+        <v>4005</v>
+      </c>
+    </row>
+    <row r="249" spans="1:35">
       <c r="A249" s="10" t="s">
         <v>3443</v>
       </c>
       <c r="W249" s="10" t="s">
+        <v>4006</v>
+      </c>
+    </row>
+    <row r="250" spans="1:35">
+      <c r="A250" s="10" t="s">
+        <v>3964</v>
+      </c>
+      <c r="W250" s="10" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="251" spans="1:35">
+      <c r="A251" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="W251" s="10" t="s">
+        <v>4007</v>
+      </c>
+    </row>
+    <row r="252" spans="1:35">
+      <c r="A252" s="15" t="s">
+        <v>3965</v>
+      </c>
+      <c r="W252" s="10" t="s">
         <v>4008</v>
       </c>
     </row>
-    <row r="250" spans="1:28">
-      <c r="A250" s="10" t="s">
+    <row r="253" spans="1:35">
+      <c r="A253" s="10" t="s">
         <v>3966</v>
       </c>
-      <c r="W250" s="10" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="251" spans="1:28">
-      <c r="A251" s="10" t="s">
-        <v>101</v>
-      </c>
-      <c r="W251" s="10" t="s">
+      <c r="W253" s="10" t="s">
         <v>4009</v>
       </c>
     </row>
-    <row r="252" spans="1:28">
-      <c r="A252" s="15" t="s">
+    <row r="254" spans="1:35">
+      <c r="A254" s="10" t="s">
         <v>3967</v>
       </c>
-      <c r="W252" s="10" t="s">
+      <c r="W254" s="10" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="255" spans="1:35">
+      <c r="A255" s="10" t="s">
+        <v>3968</v>
+      </c>
+      <c r="W255" s="10" t="s">
         <v>4010</v>
       </c>
     </row>
-    <row r="253" spans="1:28">
-      <c r="A253" s="10" t="s">
-        <v>3968</v>
-      </c>
-      <c r="W253" s="10" t="s">
+    <row r="256" spans="1:35">
+      <c r="A256" s="10" t="s">
+        <v>3969</v>
+      </c>
+      <c r="W256" s="10" t="s">
         <v>4011</v>
       </c>
     </row>
-    <row r="254" spans="1:28">
-      <c r="A254" s="10" t="s">
-        <v>3969</v>
-      </c>
-      <c r="W254" s="10" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="255" spans="1:28">
-      <c r="A255" s="10" t="s">
+    <row r="257" spans="1:47">
+      <c r="A257" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="W257" s="10" t="s">
+        <v>4012</v>
+      </c>
+    </row>
+    <row r="258" spans="1:47" ht="15">
+      <c r="A258" s="15" t="s">
         <v>3970</v>
       </c>
-      <c r="W255" s="10" t="s">
-        <v>4012</v>
-      </c>
-    </row>
-    <row r="256" spans="1:28">
-      <c r="A256" s="10" t="s">
+      <c r="W258" s="10" t="s">
+        <v>4013</v>
+      </c>
+      <c r="AT258" s="23" t="s">
+        <v>4114</v>
+      </c>
+    </row>
+    <row r="259" spans="1:47" ht="15">
+      <c r="A259" s="10" t="s">
         <v>3971</v>
       </c>
-      <c r="W256" s="10" t="s">
-        <v>4013</v>
-      </c>
-    </row>
-    <row r="257" spans="1:44">
-      <c r="A257" s="10" t="s">
-        <v>101</v>
-      </c>
-      <c r="W257" s="10" t="s">
+      <c r="W259" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="AT259" s="23" t="s">
+        <v>4115</v>
+      </c>
+    </row>
+    <row r="260" spans="1:47" ht="15">
+      <c r="A260" s="10" t="s">
+        <v>3972</v>
+      </c>
+      <c r="W260" s="10" t="s">
         <v>4014</v>
       </c>
-    </row>
-    <row r="258" spans="1:44">
-      <c r="A258" s="15" t="s">
-        <v>3972</v>
-      </c>
-      <c r="W258" s="10" t="s">
+      <c r="AT260" s="23" t="s">
+        <v>4116</v>
+      </c>
+    </row>
+    <row r="261" spans="1:47" ht="15">
+      <c r="A261" s="10" t="s">
+        <v>3973</v>
+      </c>
+      <c r="W261" s="10" t="s">
         <v>4015</v>
       </c>
-    </row>
-    <row r="259" spans="1:44">
-      <c r="A259" s="10" t="s">
-        <v>3973</v>
-      </c>
-      <c r="W259" s="10" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="260" spans="1:44">
-      <c r="A260" s="10" t="s">
-        <v>3974</v>
-      </c>
-      <c r="W260" s="10" t="s">
-        <v>4016</v>
-      </c>
-    </row>
-    <row r="261" spans="1:44">
-      <c r="A261" s="10" t="s">
-        <v>3975</v>
-      </c>
-      <c r="W261" s="10" t="s">
-        <v>4017</v>
-      </c>
-    </row>
-    <row r="262" spans="1:44">
+      <c r="AT261" s="23" t="s">
+        <v>4120</v>
+      </c>
+    </row>
+    <row r="262" spans="1:47">
       <c r="A262" s="10" t="s">
         <v>101</v>
       </c>
@@ -36276,176 +37065,205 @@
         <v>46</v>
       </c>
       <c r="AR262"/>
-    </row>
-    <row r="263" spans="1:44">
+      <c r="AU262" s="70" t="s">
+        <v>4119</v>
+      </c>
+    </row>
+    <row r="263" spans="1:47" ht="15">
       <c r="A263" s="15" t="s">
+        <v>3974</v>
+      </c>
+      <c r="W263" s="11"/>
+      <c r="AR263" s="23" t="s">
+        <v>4117</v>
+      </c>
+    </row>
+    <row r="264" spans="1:47" ht="15">
+      <c r="A264" s="10" t="s">
+        <v>3975</v>
+      </c>
+      <c r="W264" s="10" t="s">
+        <v>4016</v>
+      </c>
+      <c r="AR264" s="23" t="s">
+        <v>4118</v>
+      </c>
+    </row>
+    <row r="265" spans="1:47">
+      <c r="A265" s="10" t="s">
         <v>3976</v>
-      </c>
-      <c r="W263" s="11"/>
-    </row>
-    <row r="264" spans="1:44">
-      <c r="A264" s="10" t="s">
-        <v>3977</v>
-      </c>
-      <c r="W264" s="10" t="s">
-        <v>4018</v>
-      </c>
-    </row>
-    <row r="265" spans="1:44">
-      <c r="A265" s="10" t="s">
-        <v>3978</v>
       </c>
       <c r="W265" s="10" t="s">
         <v>922</v>
       </c>
     </row>
-    <row r="266" spans="1:44">
+    <row r="266" spans="1:47">
       <c r="A266" s="10" t="s">
+        <v>3977</v>
+      </c>
+      <c r="W266" s="10" t="s">
+        <v>4017</v>
+      </c>
+    </row>
+    <row r="267" spans="1:47">
+      <c r="A267" s="10" t="s">
+        <v>3978</v>
+      </c>
+      <c r="W267" s="10" t="s">
+        <v>4018</v>
+      </c>
+    </row>
+    <row r="268" spans="1:47">
+      <c r="A268" s="10" t="s">
         <v>3979</v>
       </c>
-      <c r="W266" s="10" t="s">
+      <c r="W268" s="10" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="269" spans="1:47">
+      <c r="A269" s="10" t="s">
+        <v>3980</v>
+      </c>
+      <c r="W269" s="10" t="s">
         <v>4019</v>
       </c>
     </row>
-    <row r="267" spans="1:44">
-      <c r="A267" s="10" t="s">
-        <v>3980</v>
-      </c>
-      <c r="W267" s="10" t="s">
+    <row r="270" spans="1:47">
+      <c r="A270" s="10" t="s">
+        <v>3981</v>
+      </c>
+      <c r="W270" s="10" t="s">
         <v>4020</v>
       </c>
     </row>
-    <row r="268" spans="1:44">
-      <c r="A268" s="10" t="s">
-        <v>3981</v>
-      </c>
-      <c r="W268" s="10" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="269" spans="1:44">
-      <c r="A269" s="10" t="s">
+    <row r="271" spans="1:47">
+      <c r="A271" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="W271" s="10" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="272" spans="1:47">
+      <c r="A272" s="10" t="s">
         <v>3982</v>
       </c>
-      <c r="W269" s="10" t="s">
+      <c r="W272" s="10" t="s">
         <v>4021</v>
       </c>
     </row>
-    <row r="270" spans="1:44">
-      <c r="A270" s="10" t="s">
+    <row r="273" spans="1:51">
+      <c r="A273" s="10" t="s">
         <v>3983</v>
       </c>
-      <c r="W270" s="10" t="s">
+      <c r="W273" s="10" t="s">
         <v>4022</v>
       </c>
     </row>
-    <row r="271" spans="1:44">
-      <c r="A271" s="10" t="s">
-        <v>101</v>
-      </c>
-      <c r="W271" s="10" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="272" spans="1:44">
-      <c r="A272" s="10" t="s">
-        <v>3984</v>
-      </c>
-      <c r="W272" s="10" t="s">
-        <v>4023</v>
-      </c>
-    </row>
-    <row r="273" spans="1:23">
-      <c r="A273" s="10" t="s">
-        <v>3985</v>
-      </c>
-      <c r="W273" s="10" t="s">
-        <v>4024</v>
-      </c>
-    </row>
-    <row r="274" spans="1:23">
+    <row r="274" spans="1:51">
       <c r="A274" s="10" t="s">
         <v>46</v>
       </c>
       <c r="W274" s="10" t="s">
-        <v>4025</v>
-      </c>
-    </row>
-    <row r="275" spans="1:23">
+        <v>4023</v>
+      </c>
+    </row>
+    <row r="275" spans="1:51">
       <c r="A275" s="11"/>
       <c r="W275" s="10" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="276" spans="1:23">
+    <row r="276" spans="1:51">
       <c r="A276" s="10" t="s">
+        <v>3984</v>
+      </c>
+    </row>
+    <row r="277" spans="1:51">
+      <c r="A277" s="10" t="s">
+        <v>3985</v>
+      </c>
+    </row>
+    <row r="278" spans="1:51" ht="15">
+      <c r="A278" s="10" t="s">
         <v>3986</v>
       </c>
-    </row>
-    <row r="277" spans="1:23">
-      <c r="A277" s="10" t="s">
-        <v>3987</v>
-      </c>
-    </row>
-    <row r="278" spans="1:23">
-      <c r="A278" s="10" t="s">
-        <v>3988</v>
-      </c>
-    </row>
-    <row r="279" spans="1:23">
+      <c r="AP278" s="86" t="s">
+        <v>4122</v>
+      </c>
+      <c r="AQ278" s="84"/>
+      <c r="AR278" s="84"/>
+      <c r="AS278" s="84"/>
+      <c r="AT278" s="84"/>
+      <c r="AU278" s="85"/>
+    </row>
+    <row r="279" spans="1:51">
       <c r="A279" s="10" t="s">
         <v>3457</v>
       </c>
     </row>
-    <row r="280" spans="1:23">
+    <row r="280" spans="1:51" ht="15">
       <c r="A280" s="10" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="281" spans="1:23">
+      <c r="AP280" s="86" t="s">
+        <v>4125</v>
+      </c>
+      <c r="AQ280" s="87"/>
+      <c r="AR280" s="87"/>
+      <c r="AS280" s="87"/>
+      <c r="AT280" s="87"/>
+      <c r="AU280" s="87"/>
+      <c r="AV280" s="87"/>
+      <c r="AW280" s="87"/>
+      <c r="AX280" s="88"/>
+      <c r="AY280" s="85"/>
+    </row>
+    <row r="281" spans="1:51">
       <c r="A281" s="10" t="s">
-        <v>3989</v>
-      </c>
-    </row>
-    <row r="282" spans="1:23">
+        <v>3987</v>
+      </c>
+    </row>
+    <row r="282" spans="1:51">
       <c r="A282" s="10" t="s">
         <v>3459</v>
       </c>
     </row>
-    <row r="283" spans="1:23">
+    <row r="283" spans="1:51">
       <c r="A283" s="10" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="284" spans="1:23">
+    <row r="284" spans="1:51">
       <c r="A284" s="11"/>
     </row>
-    <row r="285" spans="1:23">
+    <row r="285" spans="1:51">
       <c r="A285" s="10" t="s">
-        <v>3990</v>
-      </c>
-    </row>
-    <row r="286" spans="1:23">
+        <v>3988</v>
+      </c>
+    </row>
+    <row r="286" spans="1:51">
       <c r="A286" s="10" t="s">
-        <v>3991</v>
-      </c>
-    </row>
-    <row r="287" spans="1:23">
+        <v>3989</v>
+      </c>
+    </row>
+    <row r="287" spans="1:51">
       <c r="A287" s="10" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="288" spans="1:23">
+    <row r="288" spans="1:51">
       <c r="A288" s="11"/>
     </row>
     <row r="289" spans="1:1">
       <c r="A289" s="10" t="s">
-        <v>3992</v>
+        <v>3990</v>
       </c>
     </row>
     <row r="290" spans="1:1">
       <c r="A290" s="10" t="s">
-        <v>3993</v>
+        <v>3991</v>
       </c>
     </row>
     <row r="291" spans="1:1">
@@ -36458,32 +37276,32 @@
     </row>
     <row r="293" spans="1:1">
       <c r="A293" s="10" t="s">
-        <v>3994</v>
+        <v>3992</v>
       </c>
     </row>
     <row r="294" spans="1:1">
       <c r="A294" s="10" t="s">
-        <v>3995</v>
+        <v>3993</v>
       </c>
     </row>
     <row r="295" spans="1:1">
       <c r="A295" s="10" t="s">
-        <v>3996</v>
+        <v>3994</v>
       </c>
     </row>
     <row r="296" spans="1:1">
       <c r="A296" s="10" t="s">
-        <v>3997</v>
+        <v>3995</v>
       </c>
     </row>
     <row r="297" spans="1:1">
       <c r="A297" s="10" t="s">
-        <v>3998</v>
+        <v>3996</v>
       </c>
     </row>
     <row r="298" spans="1:1">
       <c r="A298" s="10" t="s">
-        <v>3999</v>
+        <v>3997</v>
       </c>
     </row>
     <row r="299" spans="1:1">
@@ -36496,47 +37314,50 @@
     </row>
     <row r="301" spans="1:1">
       <c r="A301" s="10" t="s">
-        <v>4000</v>
+        <v>3998</v>
       </c>
     </row>
     <row r="302" spans="1:1">
       <c r="A302" s="10" t="s">
-        <v>3996</v>
+        <v>3994</v>
       </c>
     </row>
     <row r="303" spans="1:1">
       <c r="A303" s="10" t="s">
-        <v>4001</v>
+        <v>3999</v>
       </c>
     </row>
     <row r="304" spans="1:1">
       <c r="A304" s="10" t="s">
-        <v>4002</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="305" spans="1:47">
       <c r="A305" s="10" t="s">
-        <v>3999</v>
-      </c>
-    </row>
-    <row r="306" spans="1:47">
+        <v>3997</v>
+      </c>
+    </row>
+    <row r="306" spans="1:47" ht="15">
       <c r="A306" s="10" t="s">
-        <v>4003</v>
-      </c>
-    </row>
-    <row r="307" spans="1:47" ht="14.4" thickBot="1">
+        <v>4001</v>
+      </c>
+      <c r="N306" s="23" t="s">
+        <v>4124</v>
+      </c>
+    </row>
+    <row r="307" spans="1:47" ht="15" thickBot="1">
       <c r="A307" s="10" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="308" spans="1:47" s="60" customFormat="1" ht="14.4" thickBot="1">
+    <row r="308" spans="1:47" s="60" customFormat="1" ht="15.75" thickBot="1">
       <c r="A308" s="59" t="s">
-        <v>4026</v>
-      </c>
-    </row>
-    <row r="309" spans="1:47">
+        <v>4123</v>
+      </c>
+    </row>
+    <row r="309" spans="1:47" ht="15">
       <c r="A309" s="8" t="s">
-        <v>4027</v>
+        <v>4024</v>
       </c>
       <c r="Z309" s="8" t="s">
         <v>3284</v>
@@ -36544,7 +37365,7 @@
     </row>
     <row r="310" spans="1:47">
       <c r="A310" s="10" t="s">
-        <v>4028</v>
+        <v>4025</v>
       </c>
       <c r="Z310" s="10" t="s">
         <v>3285</v>
@@ -36552,7 +37373,7 @@
     </row>
     <row r="311" spans="1:47">
       <c r="A311" s="10" t="s">
-        <v>4029</v>
+        <v>4026</v>
       </c>
       <c r="Z311" s="10" t="s">
         <v>3286</v>
@@ -36568,7 +37389,7 @@
     </row>
     <row r="313" spans="1:47">
       <c r="A313" s="10" t="s">
-        <v>4030</v>
+        <v>4027</v>
       </c>
       <c r="Z313" s="10" t="s">
         <v>3288</v>
@@ -36576,7 +37397,7 @@
     </row>
     <row r="314" spans="1:47">
       <c r="A314" s="10" t="s">
-        <v>4031</v>
+        <v>4028</v>
       </c>
       <c r="Z314" s="10" t="s">
         <v>101</v>
@@ -36592,7 +37413,7 @@
     </row>
     <row r="316" spans="1:47">
       <c r="A316" s="10" t="s">
-        <v>4032</v>
+        <v>4029</v>
       </c>
       <c r="Z316" s="10" t="s">
         <v>3290</v>
@@ -36600,7 +37421,7 @@
     </row>
     <row r="317" spans="1:47">
       <c r="A317" s="10" t="s">
-        <v>4033</v>
+        <v>4030</v>
       </c>
       <c r="Z317" s="10" t="s">
         <v>3291</v>
@@ -36609,7 +37430,7 @@
     </row>
     <row r="318" spans="1:47">
       <c r="A318" s="10" t="s">
-        <v>4034</v>
+        <v>4031</v>
       </c>
       <c r="Z318" s="10" t="s">
         <v>294</v>
@@ -36617,7 +37438,7 @@
     </row>
     <row r="319" spans="1:47">
       <c r="A319" s="10" t="s">
-        <v>4035</v>
+        <v>4032</v>
       </c>
       <c r="Z319" s="10" t="s">
         <v>282</v>
@@ -36625,7 +37446,7 @@
     </row>
     <row r="320" spans="1:47">
       <c r="A320" s="10" t="s">
-        <v>4036</v>
+        <v>4033</v>
       </c>
       <c r="Z320" s="10" t="s">
         <v>3292</v>
@@ -36633,7 +37454,7 @@
     </row>
     <row r="321" spans="1:26">
       <c r="A321" s="10" t="s">
-        <v>4037</v>
+        <v>4034</v>
       </c>
       <c r="Z321" s="10" t="s">
         <v>3293</v>
@@ -36641,7 +37462,7 @@
     </row>
     <row r="322" spans="1:26">
       <c r="A322" s="10" t="s">
-        <v>4038</v>
+        <v>4035</v>
       </c>
       <c r="Z322" s="10" t="s">
         <v>3294</v>
@@ -36657,7 +37478,7 @@
     </row>
     <row r="324" spans="1:26">
       <c r="A324" s="10" t="s">
-        <v>4039</v>
+        <v>4036</v>
       </c>
       <c r="Z324" s="10" t="s">
         <v>3295</v>
@@ -36665,7 +37486,7 @@
     </row>
     <row r="325" spans="1:26">
       <c r="A325" s="10" t="s">
-        <v>4040</v>
+        <v>4037</v>
       </c>
       <c r="Z325" s="10" t="s">
         <v>3296</v>
@@ -36673,7 +37494,7 @@
     </row>
     <row r="326" spans="1:26">
       <c r="A326" s="10" t="s">
-        <v>4041</v>
+        <v>4038</v>
       </c>
       <c r="Z326" s="10" t="s">
         <v>282</v>
@@ -36689,7 +37510,7 @@
     </row>
     <row r="328" spans="1:26">
       <c r="A328" s="10" t="s">
-        <v>4042</v>
+        <v>4039</v>
       </c>
       <c r="Z328" s="10" t="s">
         <v>3298</v>
@@ -36697,7 +37518,7 @@
     </row>
     <row r="329" spans="1:26">
       <c r="A329" s="10" t="s">
-        <v>4043</v>
+        <v>4040</v>
       </c>
       <c r="Z329" s="10" t="s">
         <v>3299</v>
@@ -36705,7 +37526,7 @@
     </row>
     <row r="330" spans="1:26">
       <c r="A330" s="10" t="s">
-        <v>4044</v>
+        <v>4041</v>
       </c>
       <c r="Z330" s="10" t="s">
         <v>3300</v>
@@ -36713,7 +37534,7 @@
     </row>
     <row r="331" spans="1:26">
       <c r="A331" s="10" t="s">
-        <v>4045</v>
+        <v>4042</v>
       </c>
       <c r="Z331" s="10" t="s">
         <v>3301</v>
@@ -36729,7 +37550,7 @@
     </row>
     <row r="333" spans="1:26">
       <c r="A333" s="10" t="s">
-        <v>4046</v>
+        <v>4043</v>
       </c>
       <c r="Z333" s="10" t="s">
         <v>3302</v>
@@ -36737,7 +37558,7 @@
     </row>
     <row r="334" spans="1:26">
       <c r="A334" s="10" t="s">
-        <v>4047</v>
+        <v>4044</v>
       </c>
       <c r="Z334" s="10" t="s">
         <v>294</v>
@@ -36759,7 +37580,7 @@
     </row>
     <row r="337" spans="1:26">
       <c r="A337" s="10" t="s">
-        <v>4048</v>
+        <v>4045</v>
       </c>
       <c r="Z337" s="10" t="s">
         <v>282</v>
@@ -36767,7 +37588,7 @@
     </row>
     <row r="338" spans="1:26">
       <c r="A338" s="10" t="s">
-        <v>4049</v>
+        <v>4046</v>
       </c>
       <c r="Z338" s="10" t="s">
         <v>3304</v>
@@ -36783,7 +37604,7 @@
     </row>
     <row r="340" spans="1:26">
       <c r="A340" s="10" t="s">
-        <v>4050</v>
+        <v>4047</v>
       </c>
       <c r="Z340" s="10" t="s">
         <v>294</v>
@@ -36805,17 +37626,17 @@
     </row>
     <row r="343" spans="1:26">
       <c r="A343" s="10" t="s">
-        <v>4051</v>
+        <v>4048</v>
       </c>
     </row>
     <row r="344" spans="1:26">
       <c r="A344" s="10" t="s">
-        <v>4052</v>
+        <v>4049</v>
       </c>
     </row>
     <row r="345" spans="1:26">
       <c r="A345" s="10" t="s">
-        <v>4053</v>
+        <v>4050</v>
       </c>
     </row>
     <row r="346" spans="1:26">
@@ -36828,37 +37649,37 @@
     </row>
     <row r="348" spans="1:26">
       <c r="A348" s="10" t="s">
-        <v>4054</v>
+        <v>4051</v>
       </c>
     </row>
     <row r="349" spans="1:26">
       <c r="A349" s="10" t="s">
-        <v>4055</v>
+        <v>4052</v>
       </c>
     </row>
     <row r="350" spans="1:26">
       <c r="A350" s="10" t="s">
-        <v>4056</v>
+        <v>4053</v>
       </c>
     </row>
     <row r="351" spans="1:26">
       <c r="A351" s="10" t="s">
-        <v>4057</v>
+        <v>4054</v>
       </c>
     </row>
     <row r="352" spans="1:26">
       <c r="A352" s="10" t="s">
-        <v>4058</v>
+        <v>4055</v>
       </c>
     </row>
     <row r="353" spans="1:1">
       <c r="A353" s="10" t="s">
-        <v>4059</v>
+        <v>4056</v>
       </c>
     </row>
     <row r="354" spans="1:1">
       <c r="A354" s="10" t="s">
-        <v>4058</v>
+        <v>4055</v>
       </c>
     </row>
     <row r="355" spans="1:1">
@@ -36868,22 +37689,22 @@
     </row>
     <row r="356" spans="1:1">
       <c r="A356" s="10" t="s">
-        <v>4060</v>
+        <v>4057</v>
       </c>
     </row>
     <row r="357" spans="1:1">
       <c r="A357" s="10" t="s">
-        <v>4061</v>
+        <v>4058</v>
       </c>
     </row>
     <row r="358" spans="1:1">
       <c r="A358" s="10" t="s">
-        <v>4062</v>
+        <v>4059</v>
       </c>
     </row>
     <row r="359" spans="1:1">
       <c r="A359" s="10" t="s">
-        <v>4063</v>
+        <v>4060</v>
       </c>
     </row>
     <row r="360" spans="1:1">
@@ -36896,27 +37717,27 @@
     </row>
     <row r="362" spans="1:1">
       <c r="A362" s="10" t="s">
-        <v>4064</v>
+        <v>4061</v>
       </c>
     </row>
     <row r="363" spans="1:1">
       <c r="A363" s="10" t="s">
-        <v>4065</v>
+        <v>4062</v>
       </c>
     </row>
     <row r="364" spans="1:1">
       <c r="A364" s="10" t="s">
-        <v>4066</v>
+        <v>4063</v>
       </c>
     </row>
     <row r="365" spans="1:1">
       <c r="A365" s="10" t="s">
-        <v>4067</v>
+        <v>4064</v>
       </c>
     </row>
     <row r="366" spans="1:1">
       <c r="A366" s="10" t="s">
-        <v>4068</v>
+        <v>4065</v>
       </c>
     </row>
     <row r="367" spans="1:1">
@@ -36929,22 +37750,22 @@
     </row>
     <row r="369" spans="1:1">
       <c r="A369" s="10" t="s">
-        <v>4069</v>
+        <v>4066</v>
       </c>
     </row>
     <row r="370" spans="1:1">
       <c r="A370" s="10" t="s">
-        <v>4070</v>
+        <v>4067</v>
       </c>
     </row>
     <row r="371" spans="1:1">
       <c r="A371" s="10" t="s">
-        <v>4071</v>
+        <v>4068</v>
       </c>
     </row>
     <row r="372" spans="1:1">
       <c r="A372" s="10" t="s">
-        <v>4072</v>
+        <v>4069</v>
       </c>
     </row>
     <row r="373" spans="1:1">
@@ -36954,7 +37775,7 @@
     </row>
     <row r="374" spans="1:1">
       <c r="A374" s="10" t="s">
-        <v>4073</v>
+        <v>4070</v>
       </c>
     </row>
     <row r="375" spans="1:1">
@@ -36969,12 +37790,12 @@
     </row>
     <row r="377" spans="1:1">
       <c r="A377" s="10" t="s">
-        <v>4074</v>
+        <v>4071</v>
       </c>
     </row>
     <row r="378" spans="1:1">
       <c r="A378" s="10" t="s">
-        <v>4075</v>
+        <v>4072</v>
       </c>
     </row>
     <row r="379" spans="1:1">
@@ -36987,12 +37808,12 @@
     </row>
     <row r="381" spans="1:1">
       <c r="A381" s="10" t="s">
-        <v>4076</v>
+        <v>4073</v>
       </c>
     </row>
     <row r="382" spans="1:1">
       <c r="A382" s="10" t="s">
-        <v>4077</v>
+        <v>4074</v>
       </c>
     </row>
     <row r="383" spans="1:1">
@@ -37002,22 +37823,22 @@
     </row>
     <row r="384" spans="1:1">
       <c r="A384" s="10" t="s">
-        <v>4078</v>
+        <v>4075</v>
       </c>
     </row>
     <row r="385" spans="1:1">
       <c r="A385" s="10" t="s">
-        <v>4079</v>
+        <v>4076</v>
       </c>
     </row>
     <row r="386" spans="1:1">
       <c r="A386" s="10" t="s">
-        <v>4080</v>
+        <v>4077</v>
       </c>
     </row>
     <row r="387" spans="1:1">
       <c r="A387" s="10" t="s">
-        <v>4081</v>
+        <v>4078</v>
       </c>
     </row>
     <row r="388" spans="1:1">
@@ -37030,12 +37851,12 @@
     </row>
     <row r="390" spans="1:1">
       <c r="A390" s="10" t="s">
-        <v>4082</v>
+        <v>4079</v>
       </c>
     </row>
     <row r="391" spans="1:1">
       <c r="A391" s="10" t="s">
-        <v>4083</v>
+        <v>4080</v>
       </c>
     </row>
     <row r="392" spans="1:1">
@@ -37045,7 +37866,7 @@
     </row>
     <row r="393" spans="1:1">
       <c r="A393" s="10" t="s">
-        <v>4084</v>
+        <v>4081</v>
       </c>
     </row>
     <row r="394" spans="1:1">
@@ -37055,12 +37876,12 @@
     </row>
     <row r="395" spans="1:1">
       <c r="A395" s="10" t="s">
-        <v>4078</v>
+        <v>4075</v>
       </c>
     </row>
     <row r="396" spans="1:1">
       <c r="A396" s="10" t="s">
-        <v>4079</v>
+        <v>4076</v>
       </c>
     </row>
     <row r="397" spans="1:1">
@@ -37075,22 +37896,22 @@
     </row>
     <row r="399" spans="1:1">
       <c r="A399" s="10" t="s">
-        <v>4085</v>
+        <v>4082</v>
       </c>
     </row>
     <row r="400" spans="1:1">
       <c r="A400" s="10" t="s">
-        <v>4086</v>
+        <v>4083</v>
       </c>
     </row>
     <row r="401" spans="1:1">
       <c r="A401" s="10" t="s">
-        <v>4087</v>
+        <v>4084</v>
       </c>
     </row>
     <row r="402" spans="1:1">
       <c r="A402" s="10" t="s">
-        <v>4081</v>
+        <v>4078</v>
       </c>
     </row>
     <row r="403" spans="1:1">
@@ -37100,7 +37921,7 @@
     </row>
     <row r="404" spans="1:1">
       <c r="A404" s="10" t="s">
-        <v>4088</v>
+        <v>4085</v>
       </c>
     </row>
     <row r="405" spans="1:1">
@@ -37113,17 +37934,17 @@
     </row>
     <row r="407" spans="1:1">
       <c r="A407" s="10" t="s">
-        <v>4089</v>
+        <v>4086</v>
       </c>
     </row>
     <row r="408" spans="1:1">
       <c r="A408" s="10" t="s">
-        <v>4090</v>
+        <v>4087</v>
       </c>
     </row>
     <row r="409" spans="1:1">
       <c r="A409" s="10" t="s">
-        <v>4084</v>
+        <v>4081</v>
       </c>
     </row>
     <row r="410" spans="1:1">
@@ -37133,12 +37954,12 @@
     </row>
     <row r="411" spans="1:1">
       <c r="A411" s="10" t="s">
-        <v>4091</v>
+        <v>4088</v>
       </c>
     </row>
     <row r="412" spans="1:1">
       <c r="A412" s="10" t="s">
-        <v>4079</v>
+        <v>4076</v>
       </c>
     </row>
     <row r="413" spans="1:1">
@@ -37148,7 +37969,7 @@
     </row>
     <row r="414" spans="1:1">
       <c r="A414" s="10" t="s">
-        <v>4092</v>
+        <v>4089</v>
       </c>
     </row>
     <row r="415" spans="1:1">
@@ -37158,7 +37979,7 @@
     </row>
     <row r="416" spans="1:1">
       <c r="A416" s="10" t="s">
-        <v>4093</v>
+        <v>4090</v>
       </c>
     </row>
     <row r="417" spans="1:30">
@@ -37168,17 +37989,17 @@
     </row>
     <row r="418" spans="1:30">
       <c r="A418" s="10" t="s">
-        <v>3950</v>
+        <v>3949</v>
       </c>
     </row>
     <row r="419" spans="1:30">
       <c r="A419" s="10" t="s">
-        <v>4094</v>
+        <v>4091</v>
       </c>
     </row>
     <row r="420" spans="1:30">
       <c r="A420" s="10" t="s">
-        <v>4095</v>
+        <v>4092</v>
       </c>
     </row>
     <row r="421" spans="1:30">
@@ -37188,7 +38009,7 @@
     </row>
     <row r="422" spans="1:30">
       <c r="A422" s="10" t="s">
-        <v>4096</v>
+        <v>4093</v>
       </c>
     </row>
     <row r="423" spans="1:30">
@@ -37203,20 +38024,20 @@
     </row>
     <row r="425" spans="1:30">
       <c r="A425" s="10" t="s">
-        <v>4081</v>
-      </c>
-    </row>
-    <row r="426" spans="1:30" ht="14.4" thickBot="1">
+        <v>4078</v>
+      </c>
+    </row>
+    <row r="426" spans="1:30" ht="15" thickBot="1">
       <c r="A426" s="10" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="427" spans="1:30" s="60" customFormat="1" ht="14.4" thickBot="1">
+    <row r="427" spans="1:30" s="60" customFormat="1" ht="15.75" thickBot="1">
       <c r="A427" s="59" t="s">
         <v>3306</v>
       </c>
     </row>
-    <row r="428" spans="1:30">
+    <row r="428" spans="1:30" ht="15">
       <c r="A428" s="8" t="s">
         <v>3307</v>
       </c>
@@ -37640,17 +38461,17 @@
         <v>3386</v>
       </c>
     </row>
-    <row r="484" spans="1:65" ht="14.4" thickBot="1">
+    <row r="484" spans="1:65" ht="15" thickBot="1">
       <c r="AD484" s="10" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="485" spans="1:65" s="14" customFormat="1" ht="14.4" thickBot="1">
+    <row r="485" spans="1:65" s="14" customFormat="1" ht="15.75" thickBot="1">
       <c r="A485" s="13" t="s">
         <v>3387</v>
       </c>
     </row>
-    <row r="486" spans="1:65">
+    <row r="486" spans="1:65" ht="15">
       <c r="A486" s="16" t="s">
         <v>3388</v>
       </c>
@@ -38205,17 +39026,17 @@
         <v>171</v>
       </c>
     </row>
-    <row r="531" spans="1:67" ht="14.4" thickBot="1">
+    <row r="531" spans="1:67" ht="15" thickBot="1">
       <c r="S531" s="10" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="532" spans="1:67" s="14" customFormat="1" ht="14.4" thickBot="1">
+    <row r="532" spans="1:67" s="14" customFormat="1" ht="15.75" thickBot="1">
       <c r="A532" s="13" t="s">
         <v>3465</v>
       </c>
     </row>
-    <row r="533" spans="1:67">
+    <row r="533" spans="1:67" ht="15">
       <c r="A533" s="16" t="s">
         <v>3466</v>
       </c>
@@ -39159,6 +39980,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>